<commit_message>
Refresh catalogs with enriched cosmetic descriptions
</commit_message>
<xml_diff>
--- a/catalog.xlsx
+++ b/catalog.xlsx
@@ -166,7 +166,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t xml:space="preserve">apivita-bee-sun-safe-spf50-5201279080198.jpg</t>
+          <t xml:space="preserve">sunscreens/apivita-bee-sun-safe-spf50-5201279080198.jpg</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -216,7 +216,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t xml:space="preserve">apivita-bee-sun-safe-promo-gel-spf50-5201279081119.jpg</t>
+          <t xml:space="preserve">sunscreens/apivita-bee-sun-safe-promo-gel-spf50-5201279081119.jpg</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -266,7 +266,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t xml:space="preserve">apivita-bee-sun-safe-spray-spf50-200ml-5201279080228.jpg</t>
+          <t xml:space="preserve">sunscreens/apivita-bee-sun-safe-spray-spf50-200ml-5201279080228.jpg</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -321,7 +321,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t xml:space="preserve">apivita-bee-sun-safe-promo-spf50-5201279088637.jpg</t>
+          <t xml:space="preserve">sunscreens/apivita-bee-sun-safe-promo-spf50-5201279088637.jpg</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -371,7 +371,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t xml:space="preserve">apivita-after-sun-cream-gel-100ml-5201279088460.png</t>
+          <t xml:space="preserve">sunscreens/apivita-after-sun-cream-gel-100ml-5201279088460.png</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -421,7 +421,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t xml:space="preserve">apivita-after-sun-cream-gel-200ml-5201279088453.jpg</t>
+          <t xml:space="preserve">sunscreens/apivita-after-sun-cream-gel-200ml-5201279088453.jpg</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -471,7 +471,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t xml:space="preserve">apivita-bee-sun-safe-gel-spf50-50ml-5201279080167.jpg</t>
+          <t xml:space="preserve">sunscreens/apivita-bee-sun-safe-gel-spf50-50ml-5201279080167.jpg</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -531,7 +531,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t xml:space="preserve">apivita-bee-sun-safe-spf50-golden-glow-5201279088491.jpg</t>
+          <t xml:space="preserve">sunscreens/apivita-bee-sun-safe-spf50-golden-glow-5201279088491.jpg</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -586,7 +586,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t xml:space="preserve">apivita-bee-sun-safe-dry-touch-spf50-50ml-5201279088484.jpg</t>
+          <t xml:space="preserve">sunscreens/apivita-bee-sun-safe-dry-touch-spf50-50ml-5201279088484.jpg</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -641,7 +641,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t xml:space="preserve">apivita-bee-sun-safe-lotion-spf50-5201279099503.jpg</t>
+          <t xml:space="preserve">sunscreens/apivita-bee-sun-safe-lotion-spf50-5201279099503.jpg</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -691,7 +691,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t xml:space="preserve">apivita-bee-sun-safe-spf50-100ml-5201279080662.jpg</t>
+          <t xml:space="preserve">sunscreens/apivita-bee-sun-safe-spf50-100ml-5201279080662.jpg</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -746,7 +746,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t xml:space="preserve">apivita-bee-sun-safe-spf50-200ml-5201279080235.jpg</t>
+          <t xml:space="preserve">sunscreens/apivita-bee-sun-safe-spf50-200ml-5201279080235.jpg</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -801,7 +801,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t xml:space="preserve">apivita-bee-sun-safe-anti-spot-anti-age-spf50-50ml-5201279100575.jpg</t>
+          <t xml:space="preserve">sunscreens/apivita-bee-sun-safe-anti-spot-anti-age-spf50-50ml-5201279100575.jpg</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -861,7 +861,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t xml:space="preserve">apivita-bee-sun-safe-gel-spf50-5201279080174.jpg</t>
+          <t xml:space="preserve">sunscreens/apivita-bee-sun-safe-gel-spf50-5201279080174.jpg</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -906,7 +906,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t xml:space="preserve">apivita-bee-sun-safe-gel-fresh-spf50-5201279094485.jpg</t>
+          <t xml:space="preserve">sunscreens/apivita-bee-sun-safe-gel-fresh-spf50-5201279094485.jpg</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -951,7 +951,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t xml:space="preserve">apivita-bee-sun-safe-100ml-5201279088477.jpg</t>
+          <t xml:space="preserve">sunscreens/apivita-bee-sun-safe-100ml-5201279088477.jpg</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t xml:space="preserve">apivita-bee-sun-safe-promo-beach-essentials-spf50-100ml-aftersun-5201279088668.jpg</t>
+          <t xml:space="preserve">sunscreens/apivita-bee-sun-safe-promo-beach-essentials-spf50-100ml-aftersun-5201279088668.jpg</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1046,7 +1046,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t xml:space="preserve">apivita-bee-sun-safe-spf50-50ml-5201279080181.jpg</t>
+          <t xml:space="preserve">sunscreens/apivita-bee-sun-safe-spf50-50ml-5201279080181.jpg</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1101,7 +1101,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t xml:space="preserve">apivita-bee-sun-safe-gel-spf30-50ml-5201279080150.jpg</t>
+          <t xml:space="preserve">sunscreens/apivita-bee-sun-safe-gel-spf30-50ml-5201279080150.jpg</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1156,7 +1156,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t xml:space="preserve">apivita-bee-sun-safe-dry-touch-spf50-5201279094508.jpg</t>
+          <t xml:space="preserve">sunscreens/apivita-bee-sun-safe-dry-touch-spf50-5201279094508.jpg</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1201,7 +1201,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t xml:space="preserve">apivita-bee-cream-fluid-spf50-aftersun-5201279099480.png</t>
+          <t xml:space="preserve">sunscreens/apivita-bee-cream-fluid-spf50-aftersun-5201279099480.png</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1251,7 +1251,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t xml:space="preserve">apivita-bee-sun-safe-sensitive-spf50-50ml-5201279080204.jpg</t>
+          <t xml:space="preserve">sunscreens/apivita-bee-sun-safe-sensitive-spf50-50ml-5201279080204.jpg</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1306,7 +1306,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t xml:space="preserve">apivita-bee-sun-safe-spf30-200ml-5201279080242.jpg</t>
+          <t xml:space="preserve">sunscreens/apivita-bee-sun-safe-spf30-200ml-5201279080242.jpg</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1361,7 +1361,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t xml:space="preserve">apivita-bee-sun-safe-spray-lotion-spf50-200ml-5201279080273.jpg</t>
+          <t xml:space="preserve">sunscreens/apivita-bee-sun-safe-spray-lotion-spf50-200ml-5201279080273.jpg</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -1416,7 +1416,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t xml:space="preserve">apivita-bee-sun-safe-spray-spf30-200ml-5201279080211.jpg</t>
+          <t xml:space="preserve">sunscreens/apivita-bee-sun-safe-spray-spf30-200ml-5201279080211.jpg</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -1471,7 +1471,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t xml:space="preserve">apivita-bee-sun-safe-spf50-aftersun-5201279099473.jpg</t>
+          <t xml:space="preserve">sunscreens/apivita-bee-sun-safe-spf50-aftersun-5201279099473.jpg</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -1521,7 +1521,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t xml:space="preserve">apivita-bee-sun-safe-spf30-100ml-5201279080266.jpg</t>
+          <t xml:space="preserve">sunscreens/apivita-bee-sun-safe-spf30-100ml-5201279080266.jpg</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -1576,7 +1576,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t xml:space="preserve">apivita-bee-sun-safe-promo-sensitive-spf50-aftersun-5201279099497.jpg</t>
+          <t xml:space="preserve">sunscreens/apivita-bee-sun-safe-promo-sensitive-spf50-aftersun-5201279099497.jpg</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -1626,7 +1626,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t xml:space="preserve">promo-bee-sun-safe-spf50-gel-100ml-5201279108021.jpg</t>
+          <t xml:space="preserve">sunscreens/promo-bee-sun-safe-spf50-gel-100ml-5201279108021.jpg</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -1681,7 +1681,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t xml:space="preserve">promo-bee-sun-safe-spf50-gel-100ml-5201279110543.jpg</t>
+          <t xml:space="preserve">sunscreens/promo-bee-sun-safe-spf50-gel-100ml-5201279110543.jpg</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -1736,7 +1736,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t xml:space="preserve">promo-bee-sun-safe-gel-spf50-gel-100ml-5201279108038.jpg</t>
+          <t xml:space="preserve">sunscreens/promo-bee-sun-safe-gel-spf50-gel-100ml-5201279108038.jpg</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -1791,7 +1791,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t xml:space="preserve">promo-bee-sun-safe-dry-touch-spf50-ha5-honey-repair-10ml-5201279108045.jpg</t>
+          <t xml:space="preserve">sunscreens/promo-bee-sun-safe-dry-touch-spf50-ha5-honey-repair-10ml-5201279108045.jpg</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -1841,7 +1841,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t xml:space="preserve">promo-bee-sun-safe-beach-essentials-spf50-100ml-gel-100ml-5201279108052.webp</t>
+          <t xml:space="preserve">sunscreens/promo-bee-sun-safe-beach-essentials-spf50-100ml-gel-100ml-5201279108052.webp</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -1891,7 +1891,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t xml:space="preserve">bioderma-photoderm-xdefense-ultrafluid-spf50-invisible-40ml-3701129813614.jpg</t>
+          <t xml:space="preserve">sunscreens/bioderma-photoderm-xdefense-ultrafluid-spf50-invisible-40ml-3701129813614.jpg</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -1946,7 +1946,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t xml:space="preserve">bioderma-photoderm-xdefense-ultrafluid-spf50-teinte-01-40ml-3701129813621.jpg</t>
+          <t xml:space="preserve">sunscreens/bioderma-photoderm-xdefense-ultrafluid-spf50-teinte-01-40ml-3701129813621.jpg</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2001,7 +2001,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t xml:space="preserve">bioderma-photoderm-xdefense-ultrafluid-spf50-teinte-02-40ml-3701129813638.jpg</t>
+          <t xml:space="preserve">sunscreens/bioderma-photoderm-xdefense-ultrafluid-spf50-teinte-02-40ml-3701129813638.jpg</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -2056,7 +2056,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t xml:space="preserve">bioderma-photoderm-xdefense-ultrafluid-spf50-teinte-03-40ml-2026-3701129813645.jpg</t>
+          <t xml:space="preserve">sunscreens/bioderma-photoderm-xdefense-ultrafluid-spf50-teinte-03-40ml-2026-3701129813645.jpg</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -2111,7 +2111,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t xml:space="preserve">bioderma-photoderm-xdefense-ultrafluid-spf50-teinte-04-40ml-2026-3701129813652.jpg</t>
+          <t xml:space="preserve">sunscreens/bioderma-photoderm-xdefense-ultrafluid-spf50-teinte-04-40ml-2026-3701129813652.jpg</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -2161,7 +2161,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t xml:space="preserve">bioderma-photoderm-invisible-stick-spf50-15gr-2026-3701129820674.jpg</t>
+          <t xml:space="preserve">sunscreens/bioderma-photoderm-invisible-stick-spf50-15gr-2026-3701129820674.jpg</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -2211,7 +2211,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t xml:space="preserve">bioderma-photoderm-creme-spf50-40ml-3701129803523.jpg</t>
+          <t xml:space="preserve">sunscreens/bioderma-photoderm-creme-spf50-40ml-3701129803523.jpg</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -2266,7 +2266,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t xml:space="preserve">bioderma-photoderm-aquafluide-neutre-teinte-40ml-3701129807385.jpg</t>
+          <t xml:space="preserve">sunscreens/bioderma-photoderm-aquafluide-neutre-teinte-40ml-3701129807385.jpg</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -2311,7 +2311,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t xml:space="preserve">bioderma-photoderm-nude-touch-spf50-tres-claire-40ml-3701129803455.jpg</t>
+          <t xml:space="preserve">sunscreens/bioderma-photoderm-nude-touch-spf50-tres-claire-40ml-3701129803455.jpg</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -2361,7 +2361,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t xml:space="preserve">bioderma-photoderm-nude-touch-spf50-claire-40ml-3701129803448.jpg</t>
+          <t xml:space="preserve">sunscreens/bioderma-photoderm-nude-touch-spf50-claire-40ml-3701129803448.jpg</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -2411,7 +2411,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t xml:space="preserve">bioderma-photoderm-nude-touch-spf50-doree-40ml-3701129803462.jpg</t>
+          <t xml:space="preserve">sunscreens/bioderma-photoderm-nude-touch-spf50-doree-40ml-3701129803462.jpg</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -2461,7 +2461,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t xml:space="preserve">bioderma-photoderm-spot-age-spf50-40ml-3701129803738.jpg</t>
+          <t xml:space="preserve">sunscreens/bioderma-photoderm-spot-age-spf50-40ml-3701129803738.jpg</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -2511,7 +2511,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t xml:space="preserve">bioderma-photoderm-m-spf50-claire-teinte-40ml-3701129804414.jpg</t>
+          <t xml:space="preserve">sunscreens/bioderma-photoderm-m-spf50-claire-teinte-40ml-3701129804414.jpg</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -2561,7 +2561,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t xml:space="preserve">bioderma-photoderm-m-spf50-doree-teinte-40ml-3701129803714.jpg</t>
+          <t xml:space="preserve">sunscreens/bioderma-photoderm-m-spf50-doree-teinte-40ml-3701129803714.jpg</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -2611,7 +2611,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t xml:space="preserve">bioderma-photoderm-akn-mat-spf30-teinte-40ml-3701129803691.jpg</t>
+          <t xml:space="preserve">sunscreens/bioderma-photoderm-akn-mat-spf30-teinte-40ml-3701129803691.jpg</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -2656,7 +2656,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t xml:space="preserve">bioderma-photoderm-ar-spf50-30ml-3701129803707.webp</t>
+          <t xml:space="preserve">sunscreens/bioderma-photoderm-ar-spf50-30ml-3701129803707.webp</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -2706,7 +2706,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t xml:space="preserve">bioderma-photoderm-ultra-fluid-ar-spf50-40ml-2026-3701129817957.jpg</t>
+          <t xml:space="preserve">sunscreens/bioderma-photoderm-ultra-fluid-ar-spf50-40ml-2026-3701129817957.jpg</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -2756,7 +2756,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t xml:space="preserve">bioderma-photoderm-lait-ultra-spf50-200ml-3701129803639.jpg</t>
+          <t xml:space="preserve">sunscreens/bioderma-photoderm-lait-ultra-spf50-200ml-3701129803639.jpg</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -2806,7 +2806,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t xml:space="preserve">bioderma-photoderm-brume-invisible-spf50-150ml-3701129806616.jpg</t>
+          <t xml:space="preserve">sunscreens/bioderma-photoderm-brume-invisible-spf50-150ml-3701129806616.jpg</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -2856,7 +2856,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t xml:space="preserve">bioderma-photoderm-brume-invisible-spf30-150ml-3701129806609.jpg</t>
+          <t xml:space="preserve">sunscreens/bioderma-photoderm-brume-invisible-spf30-150ml-3701129806609.jpg</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -2911,7 +2911,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t xml:space="preserve">bioderma-photoderm-family-spray-invisible-spf50-300ml-3701129807248.jpg</t>
+          <t xml:space="preserve">sunscreens/bioderma-photoderm-family-spray-invisible-spf50-300ml-3701129807248.jpg</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -2966,7 +2966,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t xml:space="preserve">bioderma-photoderm-family-spray-invisible-spf30-300ml-3701129807255.jpg</t>
+          <t xml:space="preserve">sunscreens/bioderma-photoderm-family-spray-invisible-spf30-300ml-3701129807255.jpg</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -3011,7 +3011,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t xml:space="preserve">bioderma-photoderm-eau-solaire-bronze-spf30-200ml-3701129807880.webp</t>
+          <t xml:space="preserve">sunscreens/bioderma-photoderm-eau-solaire-bronze-spf30-200ml-3701129807880.webp</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -3056,7 +3056,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t xml:space="preserve">bioderma-photoderm-eau-solaire-anti-ox-spf50-200ml-3701129807897.jpg</t>
+          <t xml:space="preserve">sunscreens/bioderma-photoderm-eau-solaire-anti-ox-spf50-200ml-3701129807897.jpg</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -3106,7 +3106,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t xml:space="preserve">bioderma-photoderm-pediatrics-mineral-spf50-50g-3701129807309.png</t>
+          <t xml:space="preserve">sunscreens/bioderma-photoderm-pediatrics-mineral-spf50-50g-3701129807309.png</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -3161,7 +3161,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t xml:space="preserve">bioderma-photoderm-pediatrics-spray-spf50-200ml-3701129807316.jpg</t>
+          <t xml:space="preserve">sunscreens/bioderma-photoderm-pediatrics-spray-spf50-200ml-3701129807316.jpg</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -3216,7 +3216,7 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t xml:space="preserve">bioderma-photoderm-pediatrics-lait-spf50-200ml-3701129807293.jpg</t>
+          <t xml:space="preserve">sunscreens/bioderma-photoderm-pediatrics-lait-spf50-200ml-3701129807293.jpg</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -3261,7 +3261,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t xml:space="preserve">bioderma-photoderm-apres-soleil-200ml-3701129803820.jpg</t>
+          <t xml:space="preserve">sunscreens/bioderma-photoderm-apres-soleil-200ml-3701129803820.jpg</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -3301,7 +3301,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t xml:space="preserve">bioderma-photoderm-apres-soleil-500ml-3701129803837.jpg</t>
+          <t xml:space="preserve">sunscreens/bioderma-photoderm-apres-soleil-500ml-3701129803837.jpg</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -3351,7 +3351,7 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm-ac-norm-sunscreen-fluid-tinted-spf50-50ml-5202888400131.jpg</t>
+          <t xml:space="preserve">sunscreens/frezyderm-ac-norm-sunscreen-fluid-tinted-spf50-50ml-5202888400131.jpg</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -3401,7 +3401,7 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm-ac-norm-sunscreen-fluid-spf50-50ml-5202888400025.jpg</t>
+          <t xml:space="preserve">sunscreens/frezyderm-ac-norm-sunscreen-fluid-spf50-50ml-5202888400025.jpg</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -3456,7 +3456,7 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm-active-sun-cream-face-spf30-50ml-5202888400087.jpg</t>
+          <t xml:space="preserve">sunscreens/frezyderm-active-sun-cream-face-spf30-50ml-5202888400087.jpg</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -3511,7 +3511,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm-active-sun-fluid-face-spf50-50ml-5202888400032.jpg</t>
+          <t xml:space="preserve">sunscreens/frezyderm-active-sun-fluid-face-spf50-50ml-5202888400032.jpg</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -3566,7 +3566,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm-active-sun-foundation-body-spf30-75ml-5202888400063.jpg</t>
+          <t xml:space="preserve">sunscreens/frezyderm-active-sun-foundation-body-spf30-75ml-5202888400063.jpg</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -3621,7 +3621,7 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm-active-sun-cream-face-spf50-50ml-5202888400094.jpg</t>
+          <t xml:space="preserve">sunscreens/frezyderm-active-sun-cream-face-spf50-50ml-5202888400094.jpg</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -3681,7 +3681,7 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm-active-sun-cream-sensitive-face-body-spf50-5202888400056.jpg</t>
+          <t xml:space="preserve">sunscreens/frezyderm-active-sun-cream-sensitive-face-body-spf50-5202888400056.jpg</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -3736,7 +3736,7 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm-active-sun-cream-tinted-face-spf50-5202888400100.jpg</t>
+          <t xml:space="preserve">sunscreens/frezyderm-active-sun-cream-tinted-face-spf50-5202888400100.jpg</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -3791,7 +3791,7 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm-active-sun-fluid-tinted-face-spf50-5202888400049.jpg</t>
+          <t xml:space="preserve">sunscreens/frezyderm-active-sun-fluid-tinted-face-spf50-5202888400049.jpg</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -3841,7 +3841,7 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm-active-sun-foundation-face-spf30-30ml-5202888400070.jpg</t>
+          <t xml:space="preserve">sunscreens/frezyderm-active-sun-foundation-face-spf30-30ml-5202888400070.jpg</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -3896,7 +3896,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm-active-sun-lipbalm-spf50-15ml-5202888400018.jpg</t>
+          <t xml:space="preserve">sunscreens/frezyderm-active-sun-lipbalm-spf50-15ml-5202888400018.jpg</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -3946,7 +3946,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm-anti-thermal-water-mist-300ml-5202888222368.jpg</t>
+          <t xml:space="preserve">sunscreens/frezyderm-anti-thermal-water-mist-300ml-5202888222368.jpg</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -3996,7 +3996,7 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm-baby-suncare-spf25-lotion-100ml-5202888221262.jpg</t>
+          <t xml:space="preserve">sunscreens/frezyderm-baby-suncare-spf25-lotion-100ml-5202888221262.jpg</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -4051,7 +4051,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm-bronze-water-color-mist-300ml-5202888222382.jpg</t>
+          <t xml:space="preserve">sunscreens/frezyderm-bronze-water-color-mist-300ml-5202888222382.jpg</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -4101,7 +4101,7 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm-infant-suncare-lotion-spf50-100ml-5202888271212.jpg</t>
+          <t xml:space="preserve">sunscreens/frezyderm-infant-suncare-lotion-spf50-100ml-5202888271212.jpg</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -4156,7 +4156,7 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm-kids-sunnip-lotion-spf50-150ml-25-5202888222436.jpg</t>
+          <t xml:space="preserve">sunscreens/frezyderm-kids-sunnip-lotion-spf50-150ml-25-5202888222436.jpg</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -4211,7 +4211,7 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm-kids-suncare-lotion-spf50-175ml-5202888222429.jpg</t>
+          <t xml:space="preserve">sunscreens/frezyderm-kids-suncare-lotion-spf50-175ml-5202888222429.jpg</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -4266,7 +4266,7 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm-kids-wetskin-spray-spf50-200ml-5202888221279.jpg</t>
+          <t xml:space="preserve">sunscreens/frezyderm-kids-wetskin-spray-spf50-200ml-5202888221279.jpg</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
@@ -4316,7 +4316,7 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm-proflamine-cream-40ml-5202888261015.jpg</t>
+          <t xml:space="preserve">sunscreens/frezyderm-proflamine-cream-40ml-5202888261015.jpg</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -4361,7 +4361,7 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm-sea-side-dry-mist-spf50-300ml-5202888222375.jpg</t>
+          <t xml:space="preserve">sunscreens/frezyderm-sea-side-dry-mist-spf50-300ml-5202888222375.jpg</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -4411,7 +4411,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm-self-tan-body-shape-150ml-5202888222283.jpg</t>
+          <t xml:space="preserve">sunscreens/frezyderm-self-tan-body-shape-150ml-5202888222283.jpg</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -4456,7 +4456,7 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm-sunscreen-after-sun-mousse-150ml-5202888102226.jpg</t>
+          <t xml:space="preserve">sunscreens/frezyderm-sunscreen-after-sun-mousse-150ml-5202888102226.jpg</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
@@ -4506,7 +4506,7 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm-sunscreen-cream-spray-kids-spf50-275ml-5202888222450.jpg</t>
+          <t xml:space="preserve">sunscreens/frezyderm-sunscreen-cream-spray-kids-spf50-275ml-5202888222450.jpg</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -4556,7 +4556,7 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm-sunscreen-on-the-move-spray-spf50-75ml-5202888222443.jpg</t>
+          <t xml:space="preserve">sunscreens/frezyderm-sunscreen-on-the-move-spray-spf50-75ml-5202888222443.jpg</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
@@ -4606,7 +4606,7 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm-sunscreen-tan-accelerator-cream-spf10-150ml-5202888102592.jpg</t>
+          <t xml:space="preserve">sunscreens/frezyderm-sunscreen-tan-accelerator-cream-spf10-150ml-5202888102592.jpg</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -4656,7 +4656,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm-sunscreen-cream-to-powder-spf50-50ml-5202888400124.jpg</t>
+          <t xml:space="preserve">sunscreens/frezyderm-sunscreen-cream-to-powder-spf50-50ml-5202888400124.jpg</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -4706,7 +4706,7 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm-sunscreen-fluid-to-powder-spf50-50ml-5202888400117.png</t>
+          <t xml:space="preserve">sunscreens/frezyderm-sunscreen-fluid-to-powder-spf50-50ml-5202888400117.png</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -4756,7 +4756,7 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm-sunscreen-invisible-spray-spf50-200ml-5202888222405.jpg</t>
+          <t xml:space="preserve">sunscreens/frezyderm-sunscreen-invisible-spray-spf50-200ml-5202888222405.jpg</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -4806,7 +4806,7 @@
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm-sunscreen-mousse-spf50-200ml-5202888222467.jpg</t>
+          <t xml:space="preserve">sunscreens/frezyderm-sunscreen-mousse-spf50-200ml-5202888222467.jpg</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
@@ -4856,7 +4856,7 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm-sunscreen-mousse-spf30-200ml-5202888222412.jpg</t>
+          <t xml:space="preserve">sunscreens/frezyderm-sunscreen-mousse-spf30-200ml-5202888222412.jpg</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
@@ -4906,7 +4906,7 @@
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm-sunscreen-spray-anti-seb-spf30-5202888102516.jpg</t>
+          <t xml:space="preserve">sunscreens/frezyderm-sunscreen-spray-anti-seb-spf30-5202888102516.jpg</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
@@ -4956,7 +4956,7 @@
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm-sunscreen-velvet-color-cream-spf50-5202888222351.jpg</t>
+          <t xml:space="preserve">sunscreens/frezyderm-sunscreen-velvet-color-cream-spf50-5202888222351.jpg</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
@@ -5006,7 +5006,7 @@
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm-sunscreen-velvet-color-cream-spf30-5202888222399.jpg</t>
+          <t xml:space="preserve">sunscreens/frezyderm-sunscreen-velvet-color-cream-spf30-5202888222399.jpg</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
@@ -5056,7 +5056,7 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm-sunscreen-velvet-cream-face-spf30-5202888222306.jpg</t>
+          <t xml:space="preserve">sunscreens/frezyderm-sunscreen-velvet-cream-face-spf30-5202888222306.jpg</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
@@ -5106,7 +5106,7 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm-sunscreen-velvet-cream-face-spf50-5202888222290.jpg</t>
+          <t xml:space="preserve">sunscreens/frezyderm-sunscreen-velvet-cream-face-spf50-5202888222290.jpg</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -5156,7 +5156,7 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm-sunscreen-velvet-lotion-body-spf50-5202888222313.jpg</t>
+          <t xml:space="preserve">sunscreens/frezyderm-sunscreen-velvet-lotion-body-spf50-5202888222313.jpg</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -5201,7 +5201,7 @@
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm-velvet-stars-cream-spf50-175ml-5202888222979.jpg</t>
+          <t xml:space="preserve">sunscreens/frezyderm-velvet-stars-cream-spf50-175ml-5202888222979.jpg</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -5251,7 +5251,7 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm-icy-after-sun-hydrogel-200ml-5202888222474.jpg</t>
+          <t xml:space="preserve">sunscreens/frezyderm-icy-after-sun-hydrogel-200ml-5202888222474.jpg</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -5299,6 +5299,11 @@
           <t xml:space="preserve">Frezyderm</t>
         </is>
       </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sunscreens/frezyderm-baby-suncare-lotion-spf50-100ml-5202888222481.jpg</t>
+        </is>
+      </c>
       <c r="I102" t="inlineStr">
         <is>
           <t xml:space="preserve">2200049766</t>
@@ -5346,7 +5351,7 @@
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm-active-sun-cream-spray-spf50-275ml-5202888400186.jpg</t>
+          <t xml:space="preserve">sunscreens/frezyderm-active-sun-cream-spray-spf50-275ml-5202888400186.jpg</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
@@ -5396,7 +5401,7 @@
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm-dry-oil-satin-stars-250ml-5202888271809.jpg</t>
+          <t xml:space="preserve">sunscreens/frezyderm-dry-oil-satin-stars-250ml-5202888271809.jpg</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
@@ -5446,7 +5451,7 @@
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm-sunscreen-stick-kids-spf50-20ml-5202888400193.jpg</t>
+          <t xml:space="preserve">sunscreens/frezyderm-sunscreen-stick-kids-spf50-20ml-5202888400193.jpg</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
@@ -5496,7 +5501,7 @@
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm-sunscreen-stick-glass-clean-spf50-20ml-5202888400223.jpg</t>
+          <t xml:space="preserve">sunscreens/frezyderm-sunscreen-stick-glass-clean-spf50-20ml-5202888400223.jpg</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -5541,7 +5546,7 @@
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm-sunscreen-anti-aging-liquid-spf50-50ml-5202888400209.png</t>
+          <t xml:space="preserve">sunscreens/frezyderm-sunscreen-anti-aging-liquid-spf50-50ml-5202888400209.png</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
@@ -5596,7 +5601,7 @@
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm-sunscreen-stick-extreme-sport-spf50-20ml-5202888400162.png</t>
+          <t xml:space="preserve">sunscreens/frezyderm-sunscreen-stick-extreme-sport-spf50-20ml-5202888400162.png</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
@@ -5651,7 +5656,7 @@
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t xml:space="preserve">fresh-line-helios-cream-face-spf50-50ml-5204989135592.png</t>
+          <t xml:space="preserve">sunscreens/fresh-line-helios-cream-face-spf50-50ml-5204989135592.png</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
@@ -5706,7 +5711,7 @@
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t xml:space="preserve">fresh-line-helios-milk-spray-spf50-150ml-5204989135615.jpg</t>
+          <t xml:space="preserve">sunscreens/fresh-line-helios-milk-spray-spf50-150ml-5204989135615.jpg</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
@@ -5756,7 +5761,7 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t xml:space="preserve">pharmasept-heliodor-after-sun-dry-oil-100ml-5205122004348.jpg</t>
+          <t xml:space="preserve">sunscreens/pharmasept-heliodor-after-sun-dry-oil-100ml-5205122004348.jpg</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
@@ -5801,7 +5806,7 @@
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t xml:space="preserve">pharmasept-heliodor-after-sun-lotion-200ml-5205122003426.jpg</t>
+          <t xml:space="preserve">sunscreens/pharmasept-heliodor-after-sun-lotion-200ml-5205122003426.jpg</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
@@ -5851,7 +5856,7 @@
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t xml:space="preserve">pharmasept-heliodor-baby-cream-spf50-100ml-5205122003297.jpg</t>
+          <t xml:space="preserve">sunscreens/pharmasept-heliodor-baby-cream-spf50-100ml-5205122003297.jpg</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
@@ -5911,7 +5916,7 @@
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t xml:space="preserve">pharmasept-heliodor-face-cream-tinted-spf30-50ml-5205122003884.jpg</t>
+          <t xml:space="preserve">sunscreens/pharmasept-heliodor-face-cream-tinted-spf30-50ml-5205122003884.jpg</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
@@ -5971,7 +5976,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t xml:space="preserve">pharmasept-heliodor-face-cream-tinted-spf50-50ml-5205122003891.png</t>
+          <t xml:space="preserve">sunscreens/pharmasept-heliodor-face-cream-tinted-spf50-50ml-5205122003891.png</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -6026,7 +6031,7 @@
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t xml:space="preserve">pharmasept-heliodor-face-cream-spf30-50ml-5205122003372.jpg</t>
+          <t xml:space="preserve">sunscreens/pharmasept-heliodor-face-cream-spf30-50ml-5205122003372.jpg</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
@@ -6081,7 +6086,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t xml:space="preserve">pharmasept-heliodor-face-cream-spf50-50ml-5205122003358.png</t>
+          <t xml:space="preserve">sunscreens/pharmasept-heliodor-face-cream-spf50-50ml-5205122003358.png</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -6136,7 +6141,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t xml:space="preserve">pharmasept-heliodor-face-body-cream-spf50-150ml-5205122003334.png</t>
+          <t xml:space="preserve">sunscreens/pharmasept-heliodor-face-body-cream-spf50-150ml-5205122003334.png</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -6191,7 +6196,7 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t xml:space="preserve">pharmasept-heliodor-face-body-spray-spf50-165gr-5205122003860.jpg</t>
+          <t xml:space="preserve">sunscreens/pharmasept-heliodor-face-body-spray-spf50-165gr-5205122003860.jpg</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
@@ -6246,7 +6251,7 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t xml:space="preserve">pharmasept-heliodor-kids-cream-spf50-150ml-5205122003310.jpg</t>
+          <t xml:space="preserve">sunscreens/pharmasept-heliodor-kids-cream-spf50-150ml-5205122003310.jpg</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
@@ -6301,7 +6306,7 @@
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t xml:space="preserve">pharmasept-heliodor-kids-spray-spf50-165gr-5205122003877.jpg</t>
+          <t xml:space="preserve">sunscreens/pharmasept-heliodor-kids-spray-spf50-165gr-5205122003877.jpg</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
@@ -6356,7 +6361,7 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t xml:space="preserve">pharmasept-heliodor-face-cream-spf50-50ml-5205122004805.png</t>
+          <t xml:space="preserve">sunscreens/pharmasept-heliodor-face-cream-spf50-50ml-5205122004805.png</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -6416,7 +6421,7 @@
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t xml:space="preserve">pharmasept-heliodor-face-cream-tinted-spf50-50ml-5205122004812.jpg</t>
+          <t xml:space="preserve">sunscreens/pharmasept-heliodor-face-cream-tinted-spf50-50ml-5205122004812.jpg</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
@@ -6471,7 +6476,7 @@
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t xml:space="preserve">korres-yoghurt-face-cream-spf50-50ml-yoghurt-5203069140747.jpg</t>
+          <t xml:space="preserve">sunscreens/korres-yoghurt-face-cream-spf50-50ml-yoghurt-5203069140747.jpg</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
@@ -6526,7 +6531,7 @@
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t xml:space="preserve">korres-yoghurt-aftersun-gel-150ml-5203069091087.jpg</t>
+          <t xml:space="preserve">sunscreens/korres-yoghurt-aftersun-gel-150ml-5203069091087.jpg</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
@@ -6571,7 +6576,7 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t xml:space="preserve">korres-yoghurt-emulsion-spf50-200ml-5203069126505.jpg</t>
+          <t xml:space="preserve">sunscreens/korres-yoghurt-emulsion-spf50-200ml-5203069126505.jpg</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
@@ -6626,7 +6631,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t xml:space="preserve">korres-yoghurt-spray-kids-spf50-150ml-5203069136238.jpg</t>
+          <t xml:space="preserve">sunscreens/korres-yoghurt-spray-kids-spf50-150ml-5203069136238.jpg</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
@@ -6676,7 +6681,7 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t xml:space="preserve">korres-yoghurt-face-spf50-50ml-5203069126413.jpg</t>
+          <t xml:space="preserve">sunscreens/korres-yoghurt-face-spf50-50ml-5203069126413.jpg</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
@@ -6736,7 +6741,7 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t xml:space="preserve">korres-yoghurt-spray-sensitive-spf50-150ml-5203069136221.jpg</t>
+          <t xml:space="preserve">sunscreens/korres-yoghurt-spray-sensitive-spf50-150ml-5203069136221.jpg</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
@@ -6786,7 +6791,7 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t xml:space="preserve">korres-red-grape-cream-spf50-50ml-day-cream-5203069141065.jpg</t>
+          <t xml:space="preserve">sunscreens/korres-red-grape-cream-spf50-50ml-day-cream-5203069141065.jpg</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -6841,7 +6846,7 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t xml:space="preserve">korres-aloe-aftersun-body-milk-150ml-5203069112218.jpg</t>
+          <t xml:space="preserve">sunscreens/korres-aloe-aftersun-body-milk-150ml-5203069112218.jpg</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
@@ -6886,7 +6891,7 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t xml:space="preserve">korres-yoghurt-face-eye-spf50-50ml-5203069126420.jpg</t>
+          <t xml:space="preserve">sunscreens/korres-yoghurt-face-eye-spf50-50ml-5203069126420.jpg</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
@@ -6941,7 +6946,7 @@
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t xml:space="preserve">korres-yoghurt-face-cream-spf30-50ml-yoghurt-5203069136245.jpg</t>
+          <t xml:space="preserve">sunscreens/korres-yoghurt-face-cream-spf30-50ml-yoghurt-5203069136245.jpg</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
@@ -6991,7 +6996,7 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t xml:space="preserve">korres-yoghurt-emulsion-spf50-150ml-5203069126499.jpg</t>
+          <t xml:space="preserve">sunscreens/korres-yoghurt-emulsion-spf50-150ml-5203069126499.jpg</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -7046,7 +7051,7 @@
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t xml:space="preserve">korres-spray-hair-sun-protection-150ml-5203069112225.jpg</t>
+          <t xml:space="preserve">sunscreens/korres-spray-hair-sun-protection-150ml-5203069112225.jpg</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
@@ -7096,7 +7101,7 @@
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t xml:space="preserve">korres-red-grape-cream-spf50-50ml-5203069113215.jpg</t>
+          <t xml:space="preserve">sunscreens/korres-red-grape-cream-spf50-50ml-5203069113215.jpg</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
@@ -7151,7 +7156,7 @@
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t xml:space="preserve">korres-red-grape-cream-spf50-5203069113239.jpg</t>
+          <t xml:space="preserve">sunscreens/korres-red-grape-cream-spf50-5203069113239.jpg</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
@@ -7196,7 +7201,7 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t xml:space="preserve">korres-yoghurt-face-eye-spf50-50ml-yoghurt-5203069136269.jpg</t>
+          <t xml:space="preserve">sunscreens/korres-yoghurt-face-eye-spf50-50ml-yoghurt-5203069136269.jpg</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
@@ -7251,7 +7256,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t xml:space="preserve">korres-red-grape-cream-spf50-glow-5203069113253.jpg</t>
+          <t xml:space="preserve">sunscreens/korres-red-grape-cream-spf50-glow-5203069113253.jpg</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -7301,7 +7306,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t xml:space="preserve">korres-yoghurt-face-cream-spf30-50ml-5203069126437.jpg</t>
+          <t xml:space="preserve">sunscreens/korres-yoghurt-face-cream-spf30-50ml-5203069126437.jpg</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -7351,7 +7356,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t xml:space="preserve">korres-yoghurt-kids-emulsion-spf50-200ml-5203069126468.jpg</t>
+          <t xml:space="preserve">sunscreens/korres-yoghurt-kids-emulsion-spf50-200ml-5203069126468.jpg</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
@@ -7411,7 +7416,7 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t xml:space="preserve">korres-yoghurt-face-cream-tinted-spf50-yoghurt-5203069140723.jpg</t>
+          <t xml:space="preserve">sunscreens/korres-yoghurt-face-cream-tinted-spf50-yoghurt-5203069140723.jpg</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -7459,6 +7464,11 @@
           <t xml:space="preserve">Korres</t>
         </is>
       </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sunscreens/korres-tinted-cream-spf30-50ml-foam-cleanser-5203069129162.jpg</t>
+        </is>
+      </c>
       <c r="I143" t="inlineStr">
         <is>
           <t xml:space="preserve">2200042153</t>
@@ -7511,7 +7521,7 @@
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t xml:space="preserve">korres-aegean-bronze-oil-spf10-150ml-5203069133640.webp</t>
+          <t xml:space="preserve">sunscreens/korres-aegean-bronze-oil-spf10-150ml-5203069133640.webp</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
@@ -7566,7 +7576,7 @@
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t xml:space="preserve">korres-yoghurt-face-tinted-spf30-50ml-5203069126451.webp</t>
+          <t xml:space="preserve">sunscreens/korres-yoghurt-face-tinted-spf30-50ml-5203069126451.webp</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
@@ -7621,7 +7631,7 @@
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t xml:space="preserve">korres-aegean-bronze-oil-spf20-150ml-5203069133657.jpg</t>
+          <t xml:space="preserve">sunscreens/korres-aegean-bronze-oil-spf20-150ml-5203069133657.jpg</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
@@ -7676,7 +7686,7 @@
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t xml:space="preserve">korres-yoghurt-spray-kids-spf50-150ml-5203069126475.jpg</t>
+          <t xml:space="preserve">sunscreens/korres-yoghurt-spray-kids-spf50-150ml-5203069126475.jpg</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
@@ -7726,7 +7736,7 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t xml:space="preserve">korres-coconut-almond-emulsion-baby-spf30-100ml-5203069090073.jpg</t>
+          <t xml:space="preserve">sunscreens/korres-coconut-almond-emulsion-baby-spf30-100ml-5203069090073.jpg</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
@@ -7781,7 +7791,7 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t xml:space="preserve">korres-sun-cream-spf50-anti-aging-anti-spot-5203069141058.jpg</t>
+          <t xml:space="preserve">sunscreens/korres-sun-cream-spf50-anti-aging-anti-spot-5203069141058.jpg</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
@@ -7836,7 +7846,7 @@
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t xml:space="preserve">korres-red-grape-face-cream-tinted-spf50-50ml-5203069136214.jpg</t>
+          <t xml:space="preserve">sunscreens/korres-red-grape-face-cream-tinted-spf50-50ml-5203069136214.jpg</t>
         </is>
       </c>
       <c r="I150" t="inlineStr">
@@ -7896,7 +7906,7 @@
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t xml:space="preserve">korres-yoghurt-spray-sensitive-spf50-150ml-5203069134128.jpg</t>
+          <t xml:space="preserve">sunscreens/korres-yoghurt-spray-sensitive-spf50-150ml-5203069134128.jpg</t>
         </is>
       </c>
       <c r="I151" t="inlineStr">
@@ -7956,7 +7966,7 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t xml:space="preserve">korres-yoghurt-face-cream-sensitive-tinted-spf30-50ml-5203069133633.jpg</t>
+          <t xml:space="preserve">sunscreens/korres-yoghurt-face-cream-sensitive-tinted-spf30-50ml-5203069133633.jpg</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
@@ -8016,7 +8026,7 @@
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t xml:space="preserve">korres-yoghurt-face-cream-sensitive-spf30-50ml-5203069133596.jpg</t>
+          <t xml:space="preserve">sunscreens/korres-yoghurt-face-cream-sensitive-spf30-50ml-5203069133596.jpg</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
@@ -8071,7 +8081,7 @@
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t xml:space="preserve">korres-yoghurt-face-tinted-spf50-50ml-5203069133626.jpg</t>
+          <t xml:space="preserve">sunscreens/korres-yoghurt-face-tinted-spf50-50ml-5203069133626.jpg</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
@@ -8131,7 +8141,7 @@
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t xml:space="preserve">korres-yoghurt-spray-sensitive-spf30-150ml-5203069133619.jpg</t>
+          <t xml:space="preserve">sunscreens/korres-yoghurt-spray-sensitive-spf30-150ml-5203069133619.jpg</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
@@ -8186,7 +8196,7 @@
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t xml:space="preserve">korres-yoghurt-emulsion-sensitive-spf30-200ml-5203069133602.jpg</t>
+          <t xml:space="preserve">sunscreens/korres-yoghurt-emulsion-sensitive-spf30-200ml-5203069133602.jpg</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
@@ -8236,7 +8246,7 @@
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t xml:space="preserve">korres-yoghurt-set-spray-emulsion-spf50-150ml-aftersun-spray-50ml-5203069140754.jpg</t>
+          <t xml:space="preserve">sunscreens/korres-yoghurt-set-spray-emulsion-spf50-150ml-aftersun-spray-50ml-5203069140754.jpg</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
@@ -8291,7 +8301,7 @@
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t xml:space="preserve">korres-yoghurt-cream-face-eye-spf50-50ml-serum-5203069140709.jpg</t>
+          <t xml:space="preserve">sunscreens/korres-yoghurt-cream-face-eye-spf50-50ml-serum-5203069140709.jpg</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
@@ -8346,7 +8356,7 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t xml:space="preserve">korres-aegean-bronze-spray-spf50-150ml-5203069139543.webp</t>
+          <t xml:space="preserve">sunscreens/korres-aegean-bronze-spray-spf50-150ml-5203069139543.webp</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
@@ -8396,7 +8406,7 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t xml:space="preserve">korres-yoghurt-face-spf30-50ml-foam-cleanser-5203069140730.jpg</t>
+          <t xml:space="preserve">sunscreens/korres-yoghurt-face-spf30-50ml-foam-cleanser-5203069140730.jpg</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
@@ -8451,7 +8461,7 @@
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t xml:space="preserve">cerave-sunscreen-fluid-dry-touch-spf50-50ml-3337875945622.jpg</t>
+          <t xml:space="preserve">sunscreens/cerave-hydrating-sunscreen-crv-oil-control-sun-spf50-50ml-enfr-3337875945622.jpg</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
@@ -8501,7 +8511,7 @@
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t xml:space="preserve">cerave-sunscreen-fluid-hydrating-spf50-50ml-3337875945660.webp</t>
+          <t xml:space="preserve">sunscreens/cerave-hydrating-sunscreen-crv-hydra-face-sun-spf50-50ml-enfr-3337875945660.webp</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
@@ -8556,7 +8566,7 @@
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t xml:space="preserve">cerave-sunscreen-lait-hydrating-spf30-177ml-3337875945790.jpg</t>
+          <t xml:space="preserve">sunscreens/cerave-hydrating-sunscreen-crv-hydra-sunscreen-sp30-177ml-enfr-3337875945790.jpg</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
@@ -8611,7 +8621,7 @@
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t xml:space="preserve">cerave-sunscreen-lait-hydrating-spf50-177ml-3337875945738.webp</t>
+          <t xml:space="preserve">sunscreens/cerave-hydrating-sunscreen-crv-hydra-sunscreen-sp50-177ml-enfr-3337875945738.webp</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
@@ -8666,7 +8676,7 @@
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t xml:space="preserve">cerave-sunscreen-lait-hydrating-spf30-75ml-3337875945820.jpg</t>
+          <t xml:space="preserve">sunscreens/cerave-hydrating-sunscreen-crv-hydra-sunscreen-spf30-75ml-enfr-3337875945820.jpg</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
@@ -8721,7 +8731,7 @@
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t xml:space="preserve">cerave-sunscreen-lait-hydrating-spf50-75ml-3337875945769.jpg</t>
+          <t xml:space="preserve">sunscreens/cerave-hydrating-sunscreen-crv-hydra-sunscreen-spf50-75ml-enfr-3337875945769.jpg</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
@@ -8776,7 +8786,7 @@
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t xml:space="preserve">la-roche-posay-anthelios-uvsport-brume-spf50-200ml-mist-3337875944960.jpg</t>
+          <t xml:space="preserve">sunscreens/la-roche-posay-body-anthelios-uvsport-mist-200ml-3337875944960.jpg</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
@@ -8826,7 +8836,7 @@
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t xml:space="preserve">la-roche-posay-anthelios-spray-spf30-shake-200ml-3337875696821.jpg</t>
+          <t xml:space="preserve">sunscreens/la-roche-posay-body-anth-spray-30-200ml-sp-purete-thermale-3337875696821.jpg</t>
         </is>
       </c>
       <c r="I168" t="inlineStr">
@@ -8876,7 +8886,7 @@
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t xml:space="preserve">la-roche-posay-anthelios-spray-spf50-shake-200ml-3337875696838.webp</t>
+          <t xml:space="preserve">sunscreens/la-roche-posay-body-anth-shaka-spray-50200ml_en-3337875696838.webp</t>
         </is>
       </c>
       <c r="I169" t="inlineStr">
@@ -8926,7 +8936,7 @@
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t xml:space="preserve">la-roche-posay-anthelios-uvair-serum-spf50-50ml-3337875932349.jpg</t>
+          <t xml:space="preserve">sunscreens/la-roche-posay-face-anthelios-uv-air-spf50-50ml-3337875932349.jpg</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
@@ -8976,7 +8986,7 @@
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t xml:space="preserve">la-roche-posay-anthelios-uvair-serum-spf50-light-50ml-3337875932301.jpg</t>
+          <t xml:space="preserve">sunscreens/la-roche-posay-face-anthelios-uv-air-tt-light-50ml-3337875932301.jpg</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
@@ -9026,7 +9036,7 @@
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t xml:space="preserve">la-roche-posay-anthelios-uvair-serum-spf50-medium-50ml-3337875932264.jpg</t>
+          <t xml:space="preserve">sunscreens/la-roche-posay-face-anthelios-uv-air-tt-medium-50ml-3337875932264.jpg</t>
         </is>
       </c>
       <c r="I172" t="inlineStr">
@@ -9076,7 +9086,7 @@
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t xml:space="preserve">la-roche-posay-anthelios-uvair-stick-spf50-10ml-3337875940412.jpg</t>
+          <t xml:space="preserve">sunscreens/la-roche-posay-face-anthelios-uv-air-stick-10g-3337875940412.jpg</t>
         </is>
       </c>
       <c r="I173" t="inlineStr">
@@ -9131,7 +9141,7 @@
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t xml:space="preserve">la-roche-posay-anthelios-uvsport-stick-spf50-10ml-3337875940399.jpg</t>
+          <t xml:space="preserve">sunscreens/la-roche-posay-face-anthelios-uv-sport-stick-10g-3337875940399.jpg</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
@@ -9181,7 +9191,7 @@
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t xml:space="preserve">la-roche-posay-anthelios-fluide-invisible-spf50-shake-50ml-3337875797580.jpg</t>
+          <t xml:space="preserve">sunscreens/la-roche-posay-face-anth-uvmune-flu-ap50-f50ml_fr-3337875797580.jpg</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
@@ -9231,7 +9241,7 @@
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t xml:space="preserve">la-roche-posay-anthelios-fluide-invisible-spf50-uvmune-promo-5201100731596.jpg</t>
+          <t xml:space="preserve">sunscreens/la-roche-posay-promo-26-anth-fluide-ap-toleriane-sen15ml-prom26-5201100731596.jpg</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
@@ -9276,7 +9286,7 @@
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t xml:space="preserve">la-roche-posay-anthelios-fluide-invisible-spf50-uvmune-50ml-3337875797597.jpg</t>
+          <t xml:space="preserve">sunscreens/la-roche-posay-face-anth-uvmune-flu-sp50-f50ml_en-3337875797597.jpg</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
@@ -9331,7 +9341,7 @@
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t xml:space="preserve">la-roche-posay-anthelios-fluide-invisible-spf50-uvmune-spot-3337875917407.jpg</t>
+          <t xml:space="preserve">sunscreens/la-roche-posay-face-ant-uvmune-fluid-pigment-spf5050ml-3337875917407.jpg</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
@@ -9376,7 +9386,7 @@
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t xml:space="preserve">la-roche-posay-anthelios-fluide-invisible-spf50-uvmune-50ml-3337875886307.jpg</t>
+          <t xml:space="preserve">sunscreens/la-roche-posay-kids-anth-uvmune-fluid-dp-spf50-50ml-3337875886307.jpg</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
@@ -9426,7 +9436,7 @@
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t xml:space="preserve">la-roche-posay-anthelios-oil-correct-gel-cream-spf50-50ml-3337875651196.jpg</t>
+          <t xml:space="preserve">sunscreens/la-roche-posay-anthelios-oil-correct-gel-cream-spf50-50ml-3337875651196.jpg</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
@@ -9481,7 +9491,7 @@
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t xml:space="preserve">la-roche-posay-anthelios-fluide-oil-control-spf50-uvmune-promo-5201100731770.jpg</t>
+          <t xml:space="preserve">sunscreens/la-roche-posay-promo-26-anth-oilcont-fl-toleriane-sen15ml-prom26-5201100731770.jpg</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
@@ -9531,7 +9541,7 @@
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t xml:space="preserve">la-roche-posay-anthelios-fluide-oil-control-spf50-uvmune-50ml-3337875847292.jpg</t>
+          <t xml:space="preserve">sunscreens/la-roche-posay-face-ant-oilcont-fl-ap50-50ml-3337875847292.jpg</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
@@ -9586,7 +9596,7 @@
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t xml:space="preserve">la-roche-posay-anthelios-fluide-teinte-spf50-shake-50ml-3337875797641.png</t>
+          <t xml:space="preserve">sunscreens/la-roche-posay-face-anth-uvmune-flu-aptt50-f50ml_en-3337875797641.png</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
@@ -9641,7 +9651,7 @@
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t xml:space="preserve">la-roche-posay-anthelios-gel-cream-oil-control-spf50-uvmune-promo-5201100731794.jpg</t>
+          <t xml:space="preserve">sunscreens/la-roche-posay-promo-26-anth-oilcont-gel-toleriane-sen15-prom26-5201100731794.jpg</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
@@ -9686,7 +9696,7 @@
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t xml:space="preserve">la-roche-posay-anthelios-lait-hydratant-spf50-uvmune-50ml-3337875888899.jpg</t>
+          <t xml:space="preserve">sunscreens/la-roche-posay-kids-anth-uvmune-dp-milk-50-75ml-3337875888899.jpg</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
@@ -9741,7 +9751,7 @@
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t xml:space="preserve">la-roche-posay-anthelios-lait-dermo-pediatrics-spf50-uvmune-250ml-3337875888851.png</t>
+          <t xml:space="preserve">sunscreens/la-roche-posay-kids-ant-uvm-milk-dp50-250ml-3337875888851.png</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
@@ -9796,7 +9806,7 @@
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t xml:space="preserve">la-roche-posay-anthelios-spray-dermo-pediatrics-spf50-uvmune-200ml-3337875886055.png</t>
+          <t xml:space="preserve">sunscreens/la-roche-posay-kids-ant-uvm-dp-spray-50-200ml-3337875886055.png</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
@@ -9846,7 +9856,7 @@
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t xml:space="preserve">la-roche-posay-anthelios-xl-brume-invisible-spf50-ultra-200ml-3337872420153.jpg</t>
+          <t xml:space="preserve">sunscreens/la-roche-posay-anth-body-mist-xl50-200ml-sp-f-3337872420153.jpg</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
@@ -9901,7 +9911,7 @@
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t xml:space="preserve">la-roche-posay-anthelios-xl-gel-cream-dry-touch-spf50-3337875546409.jpg</t>
+          <t xml:space="preserve">sunscreens/la-roche-posay-face-dtgel-uvmune-ap-50t50-3337875546409.jpg</t>
         </is>
       </c>
       <c r="I189" t="inlineStr">
@@ -9951,7 +9961,7 @@
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t xml:space="preserve">la-roche-posay-anthelios-xl-gel-cream-dry-touch-spf50-3337875545891.jpg</t>
+          <t xml:space="preserve">sunscreens/la-roche-posay-face-dtgel-uvmune-aptt-5050ml-3337875545891.jpg</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
@@ -9996,7 +10006,7 @@
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t xml:space="preserve">la-roche-posay-anthelios-100ka-med-cream-spf50-50ml-3337875798181.png</t>
+          <t xml:space="preserve">sunscreens/la-roche-posay-face-anthelios-ka-3337875798181.png</t>
         </is>
       </c>
       <c r="I191" t="inlineStr">
@@ -10046,7 +10056,7 @@
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t xml:space="preserve">la-roche-posay-anthelios-age-correct-cream-spf50-promo-5201100731619.jpg</t>
+          <t xml:space="preserve">sunscreens/la-roche-posay-promo-26-anth-age-correcthyalu-10ml-promo26-5201100731619.jpg</t>
         </is>
       </c>
       <c r="I192" t="inlineStr">
@@ -10091,7 +10101,7 @@
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t xml:space="preserve">la-roche-posay-anthelios-age-correct-cream-spf50-50ml-3337875761031.jpg</t>
+          <t xml:space="preserve">sunscreens/la-roche-posay-face-anth-uv-daily-aa-50ml-3337875761031.jpg</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
@@ -10146,7 +10156,7 @@
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t xml:space="preserve">la-roche-posay-anthelios-age-correct-teinte-cream-spf50-50ml-3337875764353.png</t>
+          <t xml:space="preserve">sunscreens/la-roche-posay-face-age-correct-tt-50ml-3337875764353.png</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
@@ -10201,7 +10211,7 @@
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t xml:space="preserve">la-roche-posay-anthelios-bebe-lait-spf50-50ml-3337872419904.jpg</t>
+          <t xml:space="preserve">sunscreens/la-roche-posay-kids-anth-dp-lait-bebe-50f50mlf-g-3337872419904.jpg</t>
         </is>
       </c>
       <c r="I195" t="inlineStr">
@@ -10251,7 +10261,7 @@
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t xml:space="preserve">la-roche-posay-anthelios-brume-invisible-spf50-75ml-3337875549530.jpg</t>
+          <t xml:space="preserve">sunscreens/la-roche-posay-anth-face-mist-xl50-75ml-ge-3337875549530.jpg</t>
         </is>
       </c>
       <c r="I196" t="inlineStr">
@@ -10306,7 +10316,7 @@
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t xml:space="preserve">la-roche-posay-anthelios-kids-lotion-wet-skin-spf50-200ml-3337875845489.jpg</t>
+          <t xml:space="preserve">sunscreens/la-roche-posay-kids-ant-wetskin-dp50-tc200ml_en-3337875845489.jpg</t>
         </is>
       </c>
       <c r="I197" t="inlineStr">
@@ -10356,7 +10366,7 @@
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t xml:space="preserve">la-roche-posay-anthelios-post-uv-exposure-lotion-200ml-3337875886024.jpg</t>
+          <t xml:space="preserve">sunscreens/la-roche-posay-after-sun-anthelios-post-uv-milky-balm-200ml-3337875886024.jpg</t>
         </is>
       </c>
       <c r="I198" t="inlineStr">
@@ -10406,7 +10416,7 @@
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t xml:space="preserve">la-roche-posay-anthelios-spray-spf50-family-300ml-3337875799348.jpg</t>
+          <t xml:space="preserve">sunscreens/la-roche-posay-body-anth-fam-spray-sp50-300ml_en-3337875799348.jpg</t>
         </is>
       </c>
       <c r="I199" t="inlineStr">
@@ -10456,7 +10466,7 @@
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t xml:space="preserve">la-roche-posay-anthelios-ultra-cream-spf50-50ml-3337875797719.jpg</t>
+          <t xml:space="preserve">sunscreens/la-roche-posay-face-ant-uvmune-ultcr-sp50t50ml_e-f-3337875797719.jpg</t>
         </is>
       </c>
       <c r="I200" t="inlineStr">
@@ -10506,7 +10516,7 @@
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t xml:space="preserve">la-roche-posay-anthelios-ultra-cream-spf50-50ml-3337875797665.png</t>
+          <t xml:space="preserve">sunscreens/la-roche-posay-face-ant-uvmune-ultcr-ap50t50ml_e-f-i-g-3337875797665.png</t>
         </is>
       </c>
       <c r="I201" t="inlineStr">
@@ -10556,7 +10566,7 @@
       </c>
       <c r="H202" t="inlineStr">
         <is>
-          <t xml:space="preserve">la-roche-posay-anthelios-ultra-lait-spf50-eco-250ml-3337875761123.jpg</t>
+          <t xml:space="preserve">sunscreens/la-roche-posay-body-anth-milk-50-tc250ml-3337875761123.jpg</t>
         </is>
       </c>
       <c r="I202" t="inlineStr">
@@ -10611,7 +10621,7 @@
       </c>
       <c r="H203" t="inlineStr">
         <is>
-          <t xml:space="preserve">la-roche-posay-anthelios-ultra-lait-spf50-wet-skin-200ml-3337875845434.jpg</t>
+          <t xml:space="preserve">sunscreens/la-roche-posay-anthelios-ultra-lait-spf50-wet-skin-200ml-3337875845434.jpg</t>
         </is>
       </c>
       <c r="I203" t="inlineStr">
@@ -10666,7 +10676,7 @@
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t xml:space="preserve">la-roche-posay-anthelios-xl-stick-sensitive-zone-spf50-9gr-3433422408616.jpg</t>
+          <t xml:space="preserve">sunscreens/la-roche-posay-anthelios-xl-stick-sensitive-zone-spf50-9gr-3433422408616.jpg</t>
         </is>
       </c>
       <c r="I204" t="inlineStr">
@@ -10716,7 +10726,7 @@
       </c>
       <c r="H205" t="inlineStr">
         <is>
-          <t xml:space="preserve">la-roche-posay-anthelios-ultra-cream-spf50-bb-50ml-3337875797689.jpg</t>
+          <t xml:space="preserve">sunscreens/la-roche-posay-face-ant-uvmune-ultcr-aptt50t50ml_en-3337875797689.jpg</t>
         </is>
       </c>
       <c r="I205" t="inlineStr">
@@ -10771,7 +10781,7 @@
       </c>
       <c r="H206" t="inlineStr">
         <is>
-          <t xml:space="preserve">la-roche-posay-anthelios-uvsport-spf50-200ml-milk-3337875945110.jpg</t>
+          <t xml:space="preserve">sunscreens/la-roche-posay-body-anthelios-uvsport-milk-200ml-3337875945110.jpg</t>
         </is>
       </c>
       <c r="I206" t="inlineStr">
@@ -10821,7 +10831,7 @@
       </c>
       <c r="H207" t="inlineStr">
         <is>
-          <t xml:space="preserve">vichy-capital-soleil-eau-spray-bronzante-spf50-200ml-3337875695152.jpg</t>
+          <t xml:space="preserve">sunscreens/vichy-body-capital-soleil-spf50-200ml-3337875695152.jpg</t>
         </is>
       </c>
       <c r="I207" t="inlineStr">
@@ -10871,7 +10881,7 @@
       </c>
       <c r="H208" t="inlineStr">
         <is>
-          <t xml:space="preserve">vichy-capital-soleil-lait-hydratant-spf50-150ml-3337875915861.jpg</t>
+          <t xml:space="preserve">sunscreens/vichy-body-capital-soleil-family-milk-spf50-150ml-3337875915861.jpg</t>
         </is>
       </c>
       <c r="I208" t="inlineStr">
@@ -10921,7 +10931,7 @@
       </c>
       <c r="H209" t="inlineStr">
         <is>
-          <t xml:space="preserve">vichy-capital-soleil-spray-bruma-spf50-200ml-3337871325770.jpg</t>
+          <t xml:space="preserve">sunscreens/vichy-body-capital-soleil-invisible-dry-touch-mist-spf50-200ml-3337871325770.jpg</t>
         </is>
       </c>
       <c r="I209" t="inlineStr">
@@ -10971,7 +10981,7 @@
       </c>
       <c r="H210" t="inlineStr">
         <is>
-          <t xml:space="preserve">vichy-capital-soleil-uvaqua-stick-spf50-9gr-3337875940993.jpg</t>
+          <t xml:space="preserve">sunscreens/vichy-face-capital-soleil-uv-aqua-stick-3337875940993.jpg</t>
         </is>
       </c>
       <c r="I210" t="inlineStr">
@@ -11021,7 +11031,7 @@
       </c>
       <c r="H211" t="inlineStr">
         <is>
-          <t xml:space="preserve">vichy-capital-soleil-after-sun-lait-apaisant-300ml-3337871322724.webp</t>
+          <t xml:space="preserve">sunscreens/vichy-capital-soleil-after-sun-lait-300ml-3337871322724.webp</t>
         </is>
       </c>
       <c r="I211" t="inlineStr">
@@ -11066,7 +11076,7 @@
       </c>
       <c r="H212" t="inlineStr">
         <is>
-          <t xml:space="preserve">vichy-capital-soleil-cream-spf50-uv-age-daily-40ml-3337875762298.jpg</t>
+          <t xml:space="preserve">sunscreens/vichy-face-capital-soleil-uv-age-spf50-40-ml-3337875762298.jpg</t>
         </is>
       </c>
       <c r="I212" t="inlineStr">
@@ -11116,7 +11126,7 @@
       </c>
       <c r="H213" t="inlineStr">
         <is>
-          <t xml:space="preserve">vichy-capital-soleil-cream-spf50-uv-age-daily-promo-5201100702299.jpg</t>
+          <t xml:space="preserve">sunscreens/vichy-capital-soleil-cream-spf50-uv-age-daily-promo-5201100702299.jpg</t>
         </is>
       </c>
       <c r="I213" t="inlineStr">
@@ -11166,7 +11176,7 @@
       </c>
       <c r="H214" t="inlineStr">
         <is>
-          <t xml:space="preserve">vichy-capital-soleil-cream-spf50-uv-age-daily-teint-40ml-3337875795265.jpg</t>
+          <t xml:space="preserve">sunscreens/vichy-face-capital-soleil-uv-age-light-shade-spf50-40-ml-3337875795265.jpg</t>
         </is>
       </c>
       <c r="I214" t="inlineStr">
@@ -11221,7 +11231,7 @@
       </c>
       <c r="H215" t="inlineStr">
         <is>
-          <t xml:space="preserve">vichy-capital-soleil-cream-spf50-uv-age-daily-teint-promo-5201100702312.jpg</t>
+          <t xml:space="preserve">sunscreens/vichy-capital-soleil-cream-spf50-uv-age-daily-teint-promo-5201100702312.jpg</t>
         </is>
       </c>
       <c r="I215" t="inlineStr">
@@ -11271,7 +11281,7 @@
       </c>
       <c r="H216" t="inlineStr">
         <is>
-          <t xml:space="preserve">vichy-capital-soleil-cream-spf50-anti-age-50ml-3337875585231.jpg</t>
+          <t xml:space="preserve">sunscreens/vichy-face-capital-soleil-anti-ageing-3in1-spf50-50ml-3337875585231.jpg</t>
         </is>
       </c>
       <c r="I216" t="inlineStr">
@@ -11326,7 +11336,7 @@
       </c>
       <c r="H217" t="inlineStr">
         <is>
-          <t xml:space="preserve">vichy-capital-soleil-cream-spf50-anti-age-promo-5201100736096.jpg</t>
+          <t xml:space="preserve">sunscreens/vichy-face-promo-anti-age-promo-box-26-5201100736096.jpg</t>
         </is>
       </c>
       <c r="I217" t="inlineStr">
@@ -11376,7 +11386,7 @@
       </c>
       <c r="H218" t="inlineStr">
         <is>
-          <t xml:space="preserve">vichy-capital-soleil-cream-spf50-dry-touch-teinte-50ml-3337871325787.jpg</t>
+          <t xml:space="preserve">sunscreens/vichy-face-capital-soleil-dry-touch-spf50-50ml-3337871325787.jpg</t>
         </is>
       </c>
       <c r="I218" t="inlineStr">
@@ -11431,7 +11441,7 @@
       </c>
       <c r="H219" t="inlineStr">
         <is>
-          <t xml:space="preserve">vichy-capital-soleil-cream-spf50-dry-touch-promo-5201100736058.jpg</t>
+          <t xml:space="preserve">sunscreens/vichy-face-promo-dry-touch-promo-box-26-5201100736058.jpg</t>
         </is>
       </c>
       <c r="I219" t="inlineStr">
@@ -11476,7 +11486,7 @@
       </c>
       <c r="H220" t="inlineStr">
         <is>
-          <t xml:space="preserve">vichy-capital-soleil-eau-spray-hydra-spf50-200ml-3337875695145.webp</t>
+          <t xml:space="preserve">sunscreens/vichy-body-capital-soleil-spf50-200ml-3337875695145.webp</t>
         </is>
       </c>
       <c r="I220" t="inlineStr">
@@ -11526,7 +11536,7 @@
       </c>
       <c r="H221" t="inlineStr">
         <is>
-          <t xml:space="preserve">vichy-capital-soleil-oil-cell-protect-spf30-200ml-3337875915915.jpg</t>
+          <t xml:space="preserve">sunscreens/vichy-capital-soleil-oil-cell-protect-spf30-200ml-3337875915915.jpg</t>
         </is>
       </c>
       <c r="I221" t="inlineStr">
@@ -11576,7 +11586,7 @@
       </c>
       <c r="H222" t="inlineStr">
         <is>
-          <t xml:space="preserve">vichy-capital-soleil-oil-spray-invisible-spf50-200ml-3337875892308.jpg</t>
+          <t xml:space="preserve">sunscreens/vichy-body-capital-soleil-spf50-200ml-3337875892308.jpg</t>
         </is>
       </c>
       <c r="I222" t="inlineStr">
@@ -11626,7 +11636,7 @@
       </c>
       <c r="H223" t="inlineStr">
         <is>
-          <t xml:space="preserve">vichy-capital-soleil-spray-anti-dehydration-spf30-200ml-3337875810890.jpg</t>
+          <t xml:space="preserve">sunscreens/vichy-body-capital-soleil-cell-protect-spray-spf30-200ml-3337875810890.jpg</t>
         </is>
       </c>
       <c r="I223" t="inlineStr">
@@ -11676,7 +11686,7 @@
       </c>
       <c r="H224" t="inlineStr">
         <is>
-          <t xml:space="preserve">vichy-capital-soleil-spray-spf50-multi-protection-200ml-3337875810869.jpg</t>
+          <t xml:space="preserve">sunscreens/vichy-body-capital-soleil-cell-protect-spray-spf50-200ml-3337875810869.jpg</t>
         </is>
       </c>
       <c r="I224" t="inlineStr">
@@ -11731,7 +11741,7 @@
       </c>
       <c r="H225" t="inlineStr">
         <is>
-          <t xml:space="preserve">vichy-capital-soleil-uv-age-fluid-spf50-40ml-teint-aftersun-5201100736072.jpg</t>
+          <t xml:space="preserve">sunscreens/vichy-face-promo-uv-age-tt-summer-box-26-5201100736072.jpg</t>
         </is>
       </c>
       <c r="I225" t="inlineStr">
@@ -11781,7 +11791,7 @@
       </c>
       <c r="H226" t="inlineStr">
         <is>
-          <t xml:space="preserve">vichy-capital-soleil-uv-age-fluid-spf50-40ml-aftersun-5201100735709.jpg</t>
+          <t xml:space="preserve">sunscreens/vichy-face-promo-uv-age-summer-box-26-5201100735709.jpg</t>
         </is>
       </c>
       <c r="I226" t="inlineStr">
@@ -11836,7 +11846,7 @@
       </c>
       <c r="H227" t="inlineStr">
         <is>
-          <t xml:space="preserve">vichy-capital-soleil-uvaqua-fluid-spf50-50ml-teinte-3337875940214.jpg</t>
+          <t xml:space="preserve">sunscreens/vichy-face-capital-soleil-uv-aqua-tinted-spf50-50ml-3337875940214.jpg</t>
         </is>
       </c>
       <c r="I227" t="inlineStr">
@@ -11886,7 +11896,7 @@
       </c>
       <c r="H228" t="inlineStr">
         <is>
-          <t xml:space="preserve">vichy-capital-soleil-uvaqua-spray-hydra-spf50-200ml-3337875940139.jpg</t>
+          <t xml:space="preserve">sunscreens/vichy-body-capital-soleil-uv-aqua-spf50-200ml-3337875940139.jpg</t>
         </is>
       </c>
       <c r="I228" t="inlineStr">
@@ -11936,7 +11946,7 @@
       </c>
       <c r="H229" t="inlineStr">
         <is>
-          <t xml:space="preserve">vichy-capital-soleil-water-fluid-spf50-uv-clear-40ml-3337875837149.webp</t>
+          <t xml:space="preserve">sunscreens/vichy-face-capital-soleil-uv-clear-spf50-40-ml-3337875837149.webp</t>
         </is>
       </c>
       <c r="I229" t="inlineStr">
@@ -11986,7 +11996,7 @@
       </c>
       <c r="H230" t="inlineStr">
         <is>
-          <t xml:space="preserve">vichy-capital-soleil-water-fluid-spf50-uv-medium-40ml-3337875915885.jpg</t>
+          <t xml:space="preserve">sunscreens/vichy-face-capital-soleil-uv-age-medium-shade-spf50-40-ml-3337875915885.jpg</t>
         </is>
       </c>
       <c r="I230" t="inlineStr">
@@ -12036,7 +12046,7 @@
       </c>
       <c r="H231" t="inlineStr">
         <is>
-          <t xml:space="preserve">vichy-capital-soleil-water-fluid-spf50-uv-age-daily-80ml-3337875914857.jpg</t>
+          <t xml:space="preserve">sunscreens/vichy-face-capital-soleil-uv-age-maxi-format-spf50-80-ml-3337875914857.jpg</t>
         </is>
       </c>
       <c r="I231" t="inlineStr">
@@ -12081,7 +12091,7 @@
       </c>
       <c r="H232" t="inlineStr">
         <is>
-          <t xml:space="preserve">vichy-ideal-soleil-aqua-spf30-pro-bronze-200ml-3337875585217.jpg</t>
+          <t xml:space="preserve">sunscreens/vichy-body-capital-soleil-spf30-200ml-3337875585217.jpg</t>
         </is>
       </c>
       <c r="I232" t="inlineStr">
@@ -12136,7 +12146,7 @@
       </c>
       <c r="H233" t="inlineStr">
         <is>
-          <t xml:space="preserve">vichy-ideal-soleil-cream-spf50-50ml-3337875419802.jpg</t>
+          <t xml:space="preserve">sunscreens/vichy-face-capital-soleil-anti-dark-spot-3in1-spf-50-50ml-3337875419802.jpg</t>
         </is>
       </c>
       <c r="I233" t="inlineStr">
@@ -12191,7 +12201,7 @@
       </c>
       <c r="H234" t="inlineStr">
         <is>
-          <t xml:space="preserve">vichy-ideal-soleil-cream-spf50-face-50ml-3337871324445.jpg</t>
+          <t xml:space="preserve">sunscreens/vichy-face-capital-soleil-velvet-cream-spf50-50ml-3337871324445.jpg</t>
         </is>
       </c>
       <c r="I234" t="inlineStr">
@@ -12241,7 +12251,7 @@
       </c>
       <c r="H235" t="inlineStr">
         <is>
-          <t xml:space="preserve">vichy-ideal-soleil-eau-spray-hydra-spf30-200ml-3337875585187.jpg</t>
+          <t xml:space="preserve">sunscreens/vichy-body-capital-soleil-spf30-200ml-3337875585187.jpg</t>
         </is>
       </c>
       <c r="I235" t="inlineStr">
@@ -12291,7 +12301,7 @@
       </c>
       <c r="H236" t="inlineStr">
         <is>
-          <t xml:space="preserve">vichy-ideal-soleil-emulsion-dry-touch-spf50-50ml-3337871323622.jpg</t>
+          <t xml:space="preserve">sunscreens/vichy-face-capital-soleil-dry-touch-spf50-50ml-3337871323622.jpg</t>
         </is>
       </c>
       <c r="I236" t="inlineStr">
@@ -12346,7 +12356,7 @@
       </c>
       <c r="H237" t="inlineStr">
         <is>
-          <t xml:space="preserve">vichy-ideal-soleil-enfant-lait-spf50-300ml-3337871323639.jpg</t>
+          <t xml:space="preserve">sunscreens/vichy-capital-soleil-lait-kids-spf50-300ml-3337871323639.jpg</t>
         </is>
       </c>
       <c r="I237" t="inlineStr">
@@ -12401,7 +12411,7 @@
       </c>
       <c r="H238" t="inlineStr">
         <is>
-          <t xml:space="preserve">vichy-ideal-soleil-lait-family-spf30-300ml-3337871321826.png</t>
+          <t xml:space="preserve">sunscreens/vichy-body-capital-soleil-family-milk-spf30-300ml-3337871321826.png</t>
         </is>
       </c>
       <c r="I238" t="inlineStr">
@@ -12456,7 +12466,7 @@
       </c>
       <c r="H239" t="inlineStr">
         <is>
-          <t xml:space="preserve">vichy-ideal-soleil-lait-sensitive-spf50-300ml-3337871322694.jpg</t>
+          <t xml:space="preserve">sunscreens/vichy-body-capital-soleil-family-milk-spf50-300ml-3337871322694.jpg</t>
         </is>
       </c>
       <c r="I239" t="inlineStr">
@@ -12511,7 +12521,7 @@
       </c>
       <c r="H240" t="inlineStr">
         <is>
-          <t xml:space="preserve">vichy-ideal-soleil-spray-enfant-spf50-200ml-3337875810838.jpg</t>
+          <t xml:space="preserve">sunscreens/vichy-capital-soleil-kids-cell-protect-uv-spray-spf50-200ml-3337875810838.jpg</t>
         </is>
       </c>
       <c r="I240" t="inlineStr">
@@ -12566,7 +12576,7 @@
       </c>
       <c r="H241" t="inlineStr">
         <is>
-          <t xml:space="preserve">vichy-ideal-soleil-stick-sensitive-spf50-9gr-30065949.jpg</t>
+          <t xml:space="preserve">sunscreens/vichy-face-capital-soleil-stick-spf50-30065949.jpg</t>
         </is>
       </c>
       <c r="I241" t="inlineStr">
@@ -12616,7 +12626,7 @@
       </c>
       <c r="H242" t="inlineStr">
         <is>
-          <t xml:space="preserve">vichy-ideal-soleil-emulsion-visage-dry-touch-spf30-50ml-3337871323196.jpg</t>
+          <t xml:space="preserve">sunscreens/vichy-face-capital-soleil-dry-touch-spf30-50ml-3337871323196.jpg</t>
         </is>
       </c>
       <c r="I242" t="inlineStr">
@@ -12671,7 +12681,7 @@
       </c>
       <c r="H243" t="inlineStr">
         <is>
-          <t xml:space="preserve">vichy-capital-soleil-cream-spf50-face-50ml-3337875940252.jpg</t>
+          <t xml:space="preserve">sunscreens/vichy-face-capital-soleil-uv-aqua-spf50-50ml-3337875940252.jpg</t>
         </is>
       </c>
       <c r="I243" t="inlineStr">
@@ -12726,7 +12736,7 @@
       </c>
       <c r="H244" t="inlineStr">
         <is>
-          <t xml:space="preserve">vichy-capital-soleil-lait-spf50-face-body-300ml-promo-5201100735686.jpg</t>
+          <t xml:space="preserve">sunscreens/vichy-body-promo-milk-promo-box-26-5201100735686.jpg</t>
         </is>
       </c>
       <c r="I244" t="inlineStr">
@@ -12771,7 +12781,7 @@
       </c>
       <c r="H245" t="inlineStr">
         <is>
-          <t xml:space="preserve">luxurious-suncare-after-sun-150ml-5205152018148.jpg</t>
+          <t xml:space="preserve">sunscreens/luxurious-suncare-after-sun-150ml-5205152018148.jpg</t>
         </is>
       </c>
       <c r="I245" t="inlineStr">
@@ -12821,7 +12831,7 @@
       </c>
       <c r="H246" t="inlineStr">
         <is>
-          <t xml:space="preserve">luxurious-suncare-body-cream-spf15-200ml-5205152018131.jpg</t>
+          <t xml:space="preserve">sunscreens/luxurious-suncare-body-cream-spf15-200ml-5205152018131.jpg</t>
         </is>
       </c>
       <c r="I246" t="inlineStr">
@@ -12876,7 +12886,7 @@
       </c>
       <c r="H247" t="inlineStr">
         <is>
-          <t xml:space="preserve">luxurious-suncare-body-cream-spf30-200ml-5205152018124.jpg</t>
+          <t xml:space="preserve">sunscreens/luxurious-suncare-body-cream-spf30-200ml-5205152018124.jpg</t>
         </is>
       </c>
       <c r="I247" t="inlineStr">
@@ -12931,7 +12941,7 @@
       </c>
       <c r="H248" t="inlineStr">
         <is>
-          <t xml:space="preserve">luxurious-suncare-body-cream-spf50-200ml-5205152018117.png</t>
+          <t xml:space="preserve">sunscreens/luxurious-suncare-body-cream-spf50-200ml-5205152018117.png</t>
         </is>
       </c>
       <c r="I248" t="inlineStr">
@@ -12986,7 +12996,7 @@
       </c>
       <c r="H249" t="inlineStr">
         <is>
-          <t xml:space="preserve">luxurious-suncare-face-body-mist-200ml-5205152018186.jpg</t>
+          <t xml:space="preserve">sunscreens/luxurious-suncare-face-body-mist-200ml-5205152018186.jpg</t>
         </is>
       </c>
       <c r="I249" t="inlineStr">
@@ -13036,7 +13046,7 @@
       </c>
       <c r="H250" t="inlineStr">
         <is>
-          <t xml:space="preserve">luxurious-suncare-face-body-mist-50ml-5205152009634.jpg</t>
+          <t xml:space="preserve">sunscreens/luxurious-suncare-face-body-mist-50ml-5205152009634.jpg</t>
         </is>
       </c>
       <c r="I250" t="inlineStr">
@@ -13081,7 +13091,7 @@
       </c>
       <c r="H251" t="inlineStr">
         <is>
-          <t xml:space="preserve">luxurious-suncare-face-spf50-75ml-5205152018155.png</t>
+          <t xml:space="preserve">sunscreens/luxurious-suncare-face-spf50-75ml-5205152018155.png</t>
         </is>
       </c>
       <c r="I251" t="inlineStr">
@@ -13126,7 +13136,7 @@
       </c>
       <c r="H252" t="inlineStr">
         <is>
-          <t xml:space="preserve">luxurious-suncare-invisible-spf30-100ml-5205152018179.jpg</t>
+          <t xml:space="preserve">sunscreens/luxurious-suncare-invisible-spf30-100ml-5205152018179.jpg</t>
         </is>
       </c>
       <c r="I252" t="inlineStr">
@@ -13171,7 +13181,7 @@
       </c>
       <c r="H253" t="inlineStr">
         <is>
-          <t xml:space="preserve">luxurious-suncare-invisible-spf30-200ml-5205152018100.jpg</t>
+          <t xml:space="preserve">sunscreens/luxurious-suncare-invisible-spf30-200ml-5205152018100.jpg</t>
         </is>
       </c>
       <c r="I253" t="inlineStr">
@@ -13216,7 +13226,7 @@
       </c>
       <c r="H254" t="inlineStr">
         <is>
-          <t xml:space="preserve">luxurious-suncare-invisible-spf50-100ml-5205152018162.webp</t>
+          <t xml:space="preserve">sunscreens/luxurious-suncare-invisible-spf50-100ml-5205152018162.webp</t>
         </is>
       </c>
       <c r="I254" t="inlineStr">
@@ -13261,7 +13271,7 @@
       </c>
       <c r="H255" t="inlineStr">
         <is>
-          <t xml:space="preserve">luxurious-suncare-invisible-spf50-200ml-5205152018094.png</t>
+          <t xml:space="preserve">sunscreens/luxurious-suncare-invisible-spf50-200ml-5205152018094.png</t>
         </is>
       </c>
       <c r="I255" t="inlineStr">
@@ -13311,7 +13321,7 @@
       </c>
       <c r="H256" t="inlineStr">
         <is>
-          <t xml:space="preserve">luxurious-suncare-self-tan-mist-200ml-5205152018209.png</t>
+          <t xml:space="preserve">sunscreens/luxurious-suncare-self-tan-mist-200ml-5205152018209.png</t>
         </is>
       </c>
       <c r="I256" t="inlineStr">
@@ -13356,7 +13366,7 @@
       </c>
       <c r="H257" t="inlineStr">
         <is>
-          <t xml:space="preserve">luxurious-suncare-dark-tan-oil-200ml-5205152018285.jpg</t>
+          <t xml:space="preserve">sunscreens/luxurious-suncare-dark-tan-oil-200ml-5205152018285.jpg</t>
         </is>
       </c>
       <c r="I257" t="inlineStr">
@@ -13406,7 +13416,7 @@
       </c>
       <c r="H258" t="inlineStr">
         <is>
-          <t xml:space="preserve">luxurious-suncare-eye-cream-spf30-15ml-5205152018216.jpg</t>
+          <t xml:space="preserve">sunscreens/luxurious-suncare-eye-cream-spf30-15ml-5205152018216.jpg</t>
         </is>
       </c>
       <c r="I258" t="inlineStr">
@@ -13461,7 +13471,7 @@
       </c>
       <c r="H259" t="inlineStr">
         <is>
-          <t xml:space="preserve">luxurious-suncare-hair-sea-mist-200ml-5205152018322.jpg</t>
+          <t xml:space="preserve">sunscreens/luxurious-suncare-hair-sea-mist-200ml-5205152018322.jpg</t>
         </is>
       </c>
       <c r="I259" t="inlineStr">
@@ -13511,7 +13521,7 @@
       </c>
       <c r="H260" t="inlineStr">
         <is>
-          <t xml:space="preserve">luxurious-suncare-lip-balm-spf30-15ml-5205152018223.jpg</t>
+          <t xml:space="preserve">sunscreens/luxurious-suncare-lip-balm-spf30-15ml-5205152018223.jpg</t>
         </is>
       </c>
       <c r="I260" t="inlineStr">
@@ -13561,7 +13571,7 @@
       </c>
       <c r="H261" t="inlineStr">
         <is>
-          <t xml:space="preserve">luxurious-suncare-monoi-oil-200ml-5205152018308.jpg</t>
+          <t xml:space="preserve">sunscreens/luxurious-suncare-monoi-oil-200ml-5205152018308.jpg</t>
         </is>
       </c>
       <c r="I261" t="inlineStr">
@@ -13601,7 +13611,7 @@
       </c>
       <c r="H262" t="inlineStr">
         <is>
-          <t xml:space="preserve">luxurious-suncare-probiotic-spf30-75ml-5205152018254.jpg</t>
+          <t xml:space="preserve">sunscreens/luxurious-suncare-probiotic-spf30-75ml-5205152018254.jpg</t>
         </is>
       </c>
       <c r="I262" t="inlineStr">
@@ -13651,7 +13661,7 @@
       </c>
       <c r="H263" t="inlineStr">
         <is>
-          <t xml:space="preserve">luxurious-suncare-serum-spf30-50ml-5205152018261.jpg</t>
+          <t xml:space="preserve">sunscreens/luxurious-suncare-serum-spf30-50ml-5205152018261.jpg</t>
         </is>
       </c>
       <c r="I263" t="inlineStr">
@@ -13696,7 +13706,7 @@
       </c>
       <c r="H264" t="inlineStr">
         <is>
-          <t xml:space="preserve">luxurious-suncare-silkcover-bronze-75ml-5205152018247.jpg</t>
+          <t xml:space="preserve">sunscreens/luxurious-suncare-silkcover-bronze-75ml-5205152018247.jpg</t>
         </is>
       </c>
       <c r="I264" t="inlineStr">
@@ -13736,7 +13746,7 @@
       </c>
       <c r="H265" t="inlineStr">
         <is>
-          <t xml:space="preserve">luxurious-suncare-silkcover-natural-75ml-5205152018230.webp</t>
+          <t xml:space="preserve">sunscreens/luxurious-suncare-silkcover-natural-75ml-5205152018230.webp</t>
         </is>
       </c>
       <c r="I265" t="inlineStr">
@@ -13781,7 +13791,7 @@
       </c>
       <c r="H266" t="inlineStr">
         <is>
-          <t xml:space="preserve">luxurious-suncare-tan-oil-spf6-200ml-5205152018292.jpg</t>
+          <t xml:space="preserve">sunscreens/luxurious-suncare-tan-oil-spf6-200ml-5205152018292.jpg</t>
         </is>
       </c>
       <c r="I266" t="inlineStr">
@@ -13826,7 +13836,7 @@
       </c>
       <c r="H267" t="inlineStr">
         <is>
-          <t xml:space="preserve">luxurious-suncare-anti-pollution-spf30-50ml-5205152018612.jpg</t>
+          <t xml:space="preserve">sunscreens/luxurious-suncare-anti-pollution-spf30-50ml-5205152018612.jpg</t>
         </is>
       </c>
       <c r="I267" t="inlineStr">
@@ -13871,7 +13881,7 @@
       </c>
       <c r="H268" t="inlineStr">
         <is>
-          <t xml:space="preserve">luxurious-suncare-instant-lifting-50ml-5205152018605.jpg</t>
+          <t xml:space="preserve">sunscreens/luxurious-suncare-instant-lifting-50ml-5205152018605.jpg</t>
         </is>
       </c>
       <c r="I268" t="inlineStr">
@@ -13916,7 +13926,7 @@
       </c>
       <c r="H269" t="inlineStr">
         <is>
-          <t xml:space="preserve">luxurious-suncare-q10-serum-50ml-5205152018278.webp</t>
+          <t xml:space="preserve">sunscreens/luxurious-suncare-q10-serum-50ml-5205152018278.webp</t>
         </is>
       </c>
       <c r="I269" t="inlineStr">
@@ -13961,7 +13971,7 @@
       </c>
       <c r="H270" t="inlineStr">
         <is>
-          <t xml:space="preserve">luxurious-suncare-bb-compact-dark-5205152018599.png</t>
+          <t xml:space="preserve">sunscreens/luxurious-suncare-bb-compact-dark-5205152018599.png</t>
         </is>
       </c>
       <c r="I270" t="inlineStr">
@@ -14001,7 +14011,7 @@
       </c>
       <c r="H271" t="inlineStr">
         <is>
-          <t xml:space="preserve">luxurious-suncare-bb-compact-light-5205152018568.jpg</t>
+          <t xml:space="preserve">sunscreens/luxurious-suncare-bb-compact-light-5205152018568.jpg</t>
         </is>
       </c>
       <c r="I271" t="inlineStr">
@@ -14041,7 +14051,7 @@
       </c>
       <c r="H272" t="inlineStr">
         <is>
-          <t xml:space="preserve">luxurious-suncare-bb-compact-medium-dark-5205152018582.jpg</t>
+          <t xml:space="preserve">sunscreens/luxurious-suncare-bb-compact-medium-dark-5205152018582.jpg</t>
         </is>
       </c>
       <c r="I272" t="inlineStr">
@@ -14081,7 +14091,7 @@
       </c>
       <c r="H273" t="inlineStr">
         <is>
-          <t xml:space="preserve">luxurious-suncare-bb-compact-medium-5205152018575.jpg</t>
+          <t xml:space="preserve">sunscreens/luxurious-suncare-bb-compact-medium-5205152018575.jpg</t>
         </is>
       </c>
       <c r="I273" t="inlineStr">
@@ -14121,7 +14131,7 @@
       </c>
       <c r="H274" t="inlineStr">
         <is>
-          <t xml:space="preserve">luxurious-suncare-stick-spf50-5205152018490.png</t>
+          <t xml:space="preserve">sunscreens/luxurious-suncare-stick-spf50-5205152018490.png</t>
         </is>
       </c>
       <c r="I274" t="inlineStr">
@@ -14166,7 +14176,7 @@
       </c>
       <c r="H275" t="inlineStr">
         <is>
-          <t xml:space="preserve">luxurious-suncare-face-spf50-body-spf15-pack-5205152018629.jpg</t>
+          <t xml:space="preserve">sunscreens/luxurious-suncare-face-spf50-body-spf15-pack-5205152018629.jpg</t>
         </is>
       </c>
       <c r="I275" t="inlineStr">
@@ -14211,7 +14221,7 @@
       </c>
       <c r="H276" t="inlineStr">
         <is>
-          <t xml:space="preserve">luxurious-suncare-face-spf50-body-spf30-pack-5205152018636.jpg</t>
+          <t xml:space="preserve">sunscreens/luxurious-suncare-face-spf50-body-spf30-pack-5205152018636.jpg</t>
         </is>
       </c>
       <c r="I276" t="inlineStr">
@@ -14256,7 +14266,7 @@
       </c>
       <c r="H277" t="inlineStr">
         <is>
-          <t xml:space="preserve">luxurious-suncare-face-spf50-body-spf50-pack-5205152018643.jpg</t>
+          <t xml:space="preserve">sunscreens/luxurious-suncare-face-spf50-body-spf50-pack-5205152018643.jpg</t>
         </is>
       </c>
       <c r="I277" t="inlineStr">
@@ -14306,7 +14316,7 @@
       </c>
       <c r="H278" t="inlineStr">
         <is>
-          <t xml:space="preserve">luxurious-suncare-hair-mist-protection-spray-pack-5205152018704.jpg</t>
+          <t xml:space="preserve">sunscreens/luxurious-suncare-hair-mist-protection-spray-pack-5205152018704.jpg</t>
         </is>
       </c>
       <c r="I278" t="inlineStr">
@@ -14341,7 +14351,7 @@
       </c>
       <c r="H279" t="inlineStr">
         <is>
-          <t xml:space="preserve">luxurious-suncare-medium-low-protection-pack-5205152018537.jpg</t>
+          <t xml:space="preserve">sunscreens/luxurious-suncare-medium-low-protection-pack-5205152018537.jpg</t>
         </is>
       </c>
       <c r="I279" t="inlineStr">
@@ -14376,7 +14386,7 @@
       </c>
       <c r="H280" t="inlineStr">
         <is>
-          <t xml:space="preserve">luxurious-suncare-travel-kit-5205152018551.jpg</t>
+          <t xml:space="preserve">sunscreens/luxurious-suncare-travel-kit-5205152018551.jpg</t>
         </is>
       </c>
       <c r="I280" t="inlineStr">
@@ -14411,7 +14421,7 @@
       </c>
       <c r="H281" t="inlineStr">
         <is>
-          <t xml:space="preserve">luxurious-suncare-high-protection-pack-5205152018506.jpg</t>
+          <t xml:space="preserve">sunscreens/luxurious-suncare-high-protection-pack-5205152018506.jpg</t>
         </is>
       </c>
       <c r="I281" t="inlineStr">
@@ -14446,7 +14456,7 @@
       </c>
       <c r="H282" t="inlineStr">
         <is>
-          <t xml:space="preserve">luxurious-suncare-towel-kit-5205152019749.jpg</t>
+          <t xml:space="preserve">sunscreens/luxurious-suncare-towel-kit-5205152019749.jpg</t>
         </is>
       </c>
       <c r="I282" t="inlineStr">
@@ -14486,7 +14496,7 @@
       </c>
       <c r="H283" t="inlineStr">
         <is>
-          <t xml:space="preserve">luxurious-suncare-protect-drops-spf50-30ml-5205152020226.jpg</t>
+          <t xml:space="preserve">sunscreens/luxurious-suncare-protect-drops-spf50-30ml-5205152020226.jpg</t>
         </is>
       </c>
       <c r="I283" t="inlineStr">
@@ -14541,7 +14551,7 @@
       </c>
       <c r="H284" t="inlineStr">
         <is>
-          <t xml:space="preserve">luxurious-suncare-hair-spray-protect-200ml-5205152018315.jpg</t>
+          <t xml:space="preserve">sunscreens/luxurious-suncare-hair-spray-protect-200ml-5205152018315.jpg</t>
         </is>
       </c>
       <c r="I284" t="inlineStr">
@@ -14586,7 +14596,7 @@
       </c>
       <c r="H285" t="inlineStr">
         <is>
-          <t xml:space="preserve">luxurious-suncare-pack-spray-spf50-invisible-hydra-5205152018544.jpg</t>
+          <t xml:space="preserve">sunscreens/luxurious-suncare-pack-spray-spf50-invisible-hydra-5205152018544.jpg</t>
         </is>
       </c>
       <c r="I285" t="inlineStr">
@@ -14631,7 +14641,7 @@
       </c>
       <c r="H286" t="inlineStr">
         <is>
-          <t xml:space="preserve">a-derma-epitheliale-a-h-ultra-cream-spf50-100ml-3282770209419.jpg</t>
+          <t xml:space="preserve">sunscreens/a-derma-epitheliale-a-h-ultra-cream-spf50-100ml-3282770209419.jpg</t>
         </is>
       </c>
       <c r="I286" t="inlineStr">
@@ -14681,7 +14691,7 @@
       </c>
       <c r="H287" t="inlineStr">
         <is>
-          <t xml:space="preserve">a-derma-epitheliale-a-h-ultra-cream-spf50-40ml-3282770209440.jpg</t>
+          <t xml:space="preserve">sunscreens/a-derma-epitheliale-a-h-ultra-cream-spf50-40ml-3282770209440.jpg</t>
         </is>
       </c>
       <c r="I287" t="inlineStr">
@@ -14726,7 +14736,7 @@
       </c>
       <c r="H288" t="inlineStr">
         <is>
-          <t xml:space="preserve">a-derma-epitheliale-a-h-ultra-reparateur-spf50-100ml-3282770398717.jpg</t>
+          <t xml:space="preserve">sunscreens/a-derma-epitheliale-a-h-ultra-reparateur-spf50-100ml-3282770398717.jpg</t>
         </is>
       </c>
       <c r="I288" t="inlineStr">
@@ -14776,7 +14786,7 @@
       </c>
       <c r="H289" t="inlineStr">
         <is>
-          <t xml:space="preserve">a-derma-exomega-control-emollient-cream-spf50-150ml-3282770397765.jpg</t>
+          <t xml:space="preserve">sunscreens/a-derma-exomega-control-emollient-cream-spf50-150ml-3282770397765.jpg</t>
         </is>
       </c>
       <c r="I289" t="inlineStr">
@@ -14831,7 +14841,7 @@
       </c>
       <c r="H290" t="inlineStr">
         <is>
-          <t xml:space="preserve">a-derma-protect-lait-kids-spf50-250ml-3282770110258.jpg</t>
+          <t xml:space="preserve">sunscreens/a-derma-protect-lait-kids-spf50-250ml-3282770110258.jpg</t>
         </is>
       </c>
       <c r="I290" t="inlineStr">
@@ -14886,7 +14896,7 @@
       </c>
       <c r="H291" t="inlineStr">
         <is>
-          <t xml:space="preserve">a-derma-protect-ac-fluid-mat-spf50-40ml-3282770072754.jpg</t>
+          <t xml:space="preserve">sunscreens/a-derma-protect-ac-fluid-mat-spf50-40ml-3282770072754.jpg</t>
         </is>
       </c>
       <c r="I291" t="inlineStr">
@@ -14936,7 +14946,7 @@
       </c>
       <c r="H292" t="inlineStr">
         <is>
-          <t xml:space="preserve">a-derma-protect-ad-cream-spf50-150ml-3282770072761.jpg</t>
+          <t xml:space="preserve">sunscreens/a-derma-protect-ad-cream-spf50-150ml-3282770072761.jpg</t>
         </is>
       </c>
       <c r="I292" t="inlineStr">
@@ -14986,7 +14996,7 @@
       </c>
       <c r="H293" t="inlineStr">
         <is>
-          <t xml:space="preserve">a-derma-protect-cream-spf50-40ml-3282770202120.jpg</t>
+          <t xml:space="preserve">sunscreens/a-derma-protect-cream-spf50-40ml-3282770202120.jpg</t>
         </is>
       </c>
       <c r="I293" t="inlineStr">
@@ -15036,7 +15046,7 @@
       </c>
       <c r="H294" t="inlineStr">
         <is>
-          <t xml:space="preserve">a-derma-protect-cream-spf50-40ml-15-3282779371629.png</t>
+          <t xml:space="preserve">sunscreens/a-derma-protect-cream-spf50-40ml-15-3282779371629.png</t>
         </is>
       </c>
       <c r="I294" t="inlineStr">
@@ -15086,7 +15096,7 @@
       </c>
       <c r="H295" t="inlineStr">
         <is>
-          <t xml:space="preserve">a-derma-protect-cream-spf50-40ml-3282770072716.jpg</t>
+          <t xml:space="preserve">sunscreens/a-derma-protect-cream-spf50-40ml-3282770072716.jpg</t>
         </is>
       </c>
       <c r="I295" t="inlineStr">
@@ -15136,7 +15146,7 @@
       </c>
       <c r="H296" t="inlineStr">
         <is>
-          <t xml:space="preserve">a-derma-protect-lait-spf50-250ml-15-3282779371643.jpg</t>
+          <t xml:space="preserve">sunscreens/a-derma-protect-lait-spf50-250ml-15-3282779371643.jpg</t>
         </is>
       </c>
       <c r="I296" t="inlineStr">
@@ -15186,7 +15196,7 @@
       </c>
       <c r="H297" t="inlineStr">
         <is>
-          <t xml:space="preserve">a-derma-protect-lait-spf50-250ml-3282770110234.jpg</t>
+          <t xml:space="preserve">sunscreens/a-derma-protect-lait-spf50-250ml-3282770110234.jpg</t>
         </is>
       </c>
       <c r="I297" t="inlineStr">
@@ -15236,7 +15246,7 @@
       </c>
       <c r="H298" t="inlineStr">
         <is>
-          <t xml:space="preserve">a-derma-protect-lait-reparateur-a-h-250ml-3282770072778.jpg</t>
+          <t xml:space="preserve">sunscreens/a-derma-protect-lait-reparateur-a-h-250ml-3282770072778.jpg</t>
         </is>
       </c>
       <c r="I298" t="inlineStr">
@@ -15281,7 +15291,7 @@
       </c>
       <c r="H299" t="inlineStr">
         <is>
-          <t xml:space="preserve">a-derma-protect-spray-spf50-200ml-3282770072730.jpg</t>
+          <t xml:space="preserve">sunscreens/a-derma-protect-spray-spf50-200ml-3282770072730.jpg</t>
         </is>
       </c>
       <c r="I299" t="inlineStr">
@@ -15336,7 +15346,7 @@
       </c>
       <c r="H300" t="inlineStr">
         <is>
-          <t xml:space="preserve">a-derma-protect-spray-kids-spf50-200ml-3282770072747.jpg</t>
+          <t xml:space="preserve">sunscreens/a-derma-protect-spray-kids-spf50-200ml-3282770072747.jpg</t>
         </is>
       </c>
       <c r="I300" t="inlineStr">
@@ -15386,7 +15396,7 @@
       </c>
       <c r="H301" t="inlineStr">
         <is>
-          <t xml:space="preserve">avene-antirougeurs-cream-jour-spf30-40ml-3282770203554.jpg</t>
+          <t xml:space="preserve">sunscreens/avene-antirougeurs-cream-jour-spf30-40ml-3282770203554.jpg</t>
         </is>
       </c>
       <c r="I301" t="inlineStr">
@@ -15431,7 +15441,7 @@
       </c>
       <c r="H302" t="inlineStr">
         <is>
-          <t xml:space="preserve">avene-antirougeurs-emulsion-jour-spf30-40ml-3282770203523.jpg</t>
+          <t xml:space="preserve">sunscreens/avene-antirougeurs-emulsion-jour-spf30-40ml-3282770203523.jpg</t>
         </is>
       </c>
       <c r="I302" t="inlineStr">
@@ -15476,7 +15486,7 @@
       </c>
       <c r="H303" t="inlineStr">
         <is>
-          <t xml:space="preserve">avene-antirougeurs-rosamax-soin-spf50-30ml-3282770395235.jpg</t>
+          <t xml:space="preserve">sunscreens/avene-antirougeurs-rosamax-soin-spf50-30ml-3282770395235.jpg</t>
         </is>
       </c>
       <c r="I303" t="inlineStr">
@@ -15526,7 +15536,7 @@
       </c>
       <c r="H304" t="inlineStr">
         <is>
-          <t xml:space="preserve">avene-cicalfate-cream-reparateur-spf50-30ml-3282770394467.jpg</t>
+          <t xml:space="preserve">sunscreens/avene-cicalfate-cream-reparateur-spf50-30ml-3282770394467.jpg</t>
         </is>
       </c>
       <c r="I304" t="inlineStr">
@@ -15581,7 +15591,7 @@
       </c>
       <c r="H305" t="inlineStr">
         <is>
-          <t xml:space="preserve">avene-cleanance-solaire-cream-spf50-50ml-color-3282770149562.jpg</t>
+          <t xml:space="preserve">sunscreens/avene-cleanance-solaire-cream-spf50-50ml-color-3282770149562.jpg</t>
         </is>
       </c>
       <c r="I305" t="inlineStr">
@@ -15631,7 +15641,7 @@
       </c>
       <c r="H306" t="inlineStr">
         <is>
-          <t xml:space="preserve">avene-cleanance-ultra-leger-cream-spf50-3282770149548.jpg</t>
+          <t xml:space="preserve">sunscreens/avene-cleanance-ultra-leger-cream-spf50-3282770149548.jpg</t>
         </is>
       </c>
       <c r="I306" t="inlineStr">
@@ -15676,7 +15686,7 @@
       </c>
       <c r="H307" t="inlineStr">
         <is>
-          <t xml:space="preserve">avene-compact-dore-haute-protection-spf50-10gr-3282770100242.jpg</t>
+          <t xml:space="preserve">sunscreens/avene-compact-dore-haute-protection-spf50-10gr-3282770100242.jpg</t>
         </is>
       </c>
       <c r="I307" t="inlineStr">
@@ -15726,7 +15736,7 @@
       </c>
       <c r="H308" t="inlineStr">
         <is>
-          <t xml:space="preserve">avene-compact-sable-spf50-10gr-3282770100228.jpg</t>
+          <t xml:space="preserve">sunscreens/avene-compact-sable-spf50-10gr-3282770100228.jpg</t>
         </is>
       </c>
       <c r="I308" t="inlineStr">
@@ -15776,7 +15786,7 @@
       </c>
       <c r="H309" t="inlineStr">
         <is>
-          <t xml:space="preserve">avene-couvrance-compact-confort-5-soleil-spf30-3282770082357.jpg</t>
+          <t xml:space="preserve">sunscreens/avene-couvrance-compact-confort-5-soleil-spf30-3282770082357.jpg</t>
         </is>
       </c>
       <c r="I309" t="inlineStr">
@@ -15821,7 +15831,7 @@
       </c>
       <c r="H310" t="inlineStr">
         <is>
-          <t xml:space="preserve">avene-eau-thermale-lait-solaire-spf50-250ml-3282770396881.jpg</t>
+          <t xml:space="preserve">sunscreens/avene-eau-thermale-lait-solaire-spf50-250ml-3282770396881.jpg</t>
         </is>
       </c>
       <c r="I310" t="inlineStr">
@@ -15926,7 +15936,7 @@
       </c>
       <c r="H312" t="inlineStr">
         <is>
-          <t xml:space="preserve">avene-fluid-antiage-spf50-triasorb-40ml-3282770396300.png</t>
+          <t xml:space="preserve">sunscreens/avene-fluid-antiage-spf50-triasorb-40ml-3282770396300.png</t>
         </is>
       </c>
       <c r="I312" t="inlineStr">
@@ -15981,7 +15991,7 @@
       </c>
       <c r="H313" t="inlineStr">
         <is>
-          <t xml:space="preserve">avene-fluid-anti-pigment-spf50-teinte-triasorb-40ml-3282770397451.jpg</t>
+          <t xml:space="preserve">sunscreens/avene-fluid-anti-pigment-spf50-teinte-triasorb-40ml-3282770397451.jpg</t>
         </is>
       </c>
       <c r="I313" t="inlineStr">
@@ -16031,7 +16041,7 @@
       </c>
       <c r="H314" t="inlineStr">
         <is>
-          <t xml:space="preserve">avene-haute-protection-brume-oil-spf30-150ml-3282770114669.jpg</t>
+          <t xml:space="preserve">sunscreens/avene-haute-protection-brume-oil-spf30-150ml-3282770114669.jpg</t>
         </is>
       </c>
       <c r="I314" t="inlineStr">
@@ -16081,7 +16091,7 @@
       </c>
       <c r="H315" t="inlineStr">
         <is>
-          <t xml:space="preserve">avene-haute-protection-spray-spf30-antioxydant-200ml-3282779402927.jpg</t>
+          <t xml:space="preserve">sunscreens/avene-haute-protection-spray-spf30-antioxydant-200ml-3282779402927.jpg</t>
         </is>
       </c>
       <c r="I315" t="inlineStr">
@@ -16131,7 +16141,7 @@
       </c>
       <c r="H316" t="inlineStr">
         <is>
-          <t xml:space="preserve">avene-haute-protection-spray-invisible-spf30-200ml-3282770392999.jpg</t>
+          <t xml:space="preserve">sunscreens/avene-haute-protection-spray-invisible-spf30-200ml-3282770392999.jpg</t>
         </is>
       </c>
       <c r="I316" t="inlineStr">
@@ -16181,7 +16191,7 @@
       </c>
       <c r="H317" t="inlineStr">
         <is>
-          <t xml:space="preserve">avene-haute-protection-spray-invisible-spf50-200ml-3282770396331.jpg</t>
+          <t xml:space="preserve">sunscreens/avene-haute-protection-spray-invisible-spf50-200ml-3282770396331.jpg</t>
         </is>
       </c>
       <c r="I317" t="inlineStr">
@@ -16231,7 +16241,7 @@
       </c>
       <c r="H318" t="inlineStr">
         <is>
-          <t xml:space="preserve">avene-huile-fini-satine-spf30-200ml-3282770389623.jpg</t>
+          <t xml:space="preserve">sunscreens/avene-huile-fini-satine-spf30-200ml-3282770389623.jpg</t>
         </is>
       </c>
       <c r="I318" t="inlineStr">
@@ -16286,7 +16296,7 @@
       </c>
       <c r="H319" t="inlineStr">
         <is>
-          <t xml:space="preserve">avene-reflexe-solaire-cream-spf50-family-30ml-3282770388961.jpg</t>
+          <t xml:space="preserve">sunscreens/avene-reflexe-solaire-cream-spf50-family-30ml-3282770388961.jpg</t>
         </is>
       </c>
       <c r="I319" t="inlineStr">
@@ -16336,7 +16346,7 @@
       </c>
       <c r="H320" t="inlineStr">
         <is>
-          <t xml:space="preserve">avene-sun-skin-protect-cream-spf50-50ml-blue-light-3282770149487.jpg</t>
+          <t xml:space="preserve">sunscreens/avene-sun-skin-protect-cream-spf50-50ml-blue-light-3282770149487.jpg</t>
         </is>
       </c>
       <c r="I320" t="inlineStr">
@@ -16386,7 +16396,7 @@
       </c>
       <c r="H321" t="inlineStr">
         <is>
-          <t xml:space="preserve">avene-sun-skin-protect-cream-spf50-blue-light-3282770149494.jpg</t>
+          <t xml:space="preserve">sunscreens/avene-sun-skin-protect-cream-spf50-blue-light-3282770149494.jpg</t>
         </is>
       </c>
       <c r="I321" t="inlineStr">
@@ -16431,7 +16441,7 @@
       </c>
       <c r="H322" t="inlineStr">
         <is>
-          <t xml:space="preserve">avene-solaire-anti-age-spf50-teinte-50ml-3282770203165.jpg</t>
+          <t xml:space="preserve">sunscreens/avene-solaire-anti-age-spf50-teinte-50ml-3282770203165.jpg</t>
         </is>
       </c>
       <c r="I322" t="inlineStr">
@@ -16481,7 +16491,7 @@
       </c>
       <c r="H323" t="inlineStr">
         <is>
-          <t xml:space="preserve">avene-sunsimed-ka-cream-uvb-uva-80ml-3282770392760.jpg</t>
+          <t xml:space="preserve">sunscreens/avene-sunsimed-ka-cream-uvb-uva-80ml-3282770392760.jpg</t>
         </is>
       </c>
       <c r="I323" t="inlineStr">
@@ -16526,7 +16536,7 @@
       </c>
       <c r="H324" t="inlineStr">
         <is>
-          <t xml:space="preserve">avene-sunsimed-cream-pigment-uvb-uva-80ml-3282770392791.jpg</t>
+          <t xml:space="preserve">sunscreens/avene-sunsimed-cream-pigment-uvb-uva-80ml-3282770392791.jpg</t>
         </is>
       </c>
       <c r="I324" t="inlineStr">
@@ -16576,7 +16586,7 @@
       </c>
       <c r="H325" t="inlineStr">
         <is>
-          <t xml:space="preserve">avene-tres-haute-protection-lait-enfant-spf50-250ml-3282770202106.jpg</t>
+          <t xml:space="preserve">sunscreens/avene-tres-haute-protection-lait-enfant-spf50-250ml-3282770202106.jpg</t>
         </is>
       </c>
       <c r="I325" t="inlineStr">
@@ -16631,7 +16641,7 @@
       </c>
       <c r="H326" t="inlineStr">
         <is>
-          <t xml:space="preserve">avene-tres-haute-protection-stick-spf50-8gr-zone-sensible-3282770204803.jpg</t>
+          <t xml:space="preserve">sunscreens/avene-tres-haute-protection-stick-spf50-8gr-zone-sensible-3282770204803.jpg</t>
         </is>
       </c>
       <c r="I326" t="inlineStr">
@@ -16686,7 +16696,7 @@
       </c>
       <c r="H327" t="inlineStr">
         <is>
-          <t xml:space="preserve">avene-tres-haute-protection-enfant-spray-spf50-200ml-3282770202090.jpg</t>
+          <t xml:space="preserve">sunscreens/avene-tres-haute-protection-enfant-spray-spf50-200ml-3282770202090.jpg</t>
         </is>
       </c>
       <c r="I327" t="inlineStr">
@@ -16741,7 +16751,7 @@
       </c>
       <c r="H328" t="inlineStr">
         <is>
-          <t xml:space="preserve">avene-tres-haute-protection-family-spray-spf50-400ml-3282770396324.jpg</t>
+          <t xml:space="preserve">sunscreens/avene-tres-haute-protection-family-spray-spf50-400ml-3282770396324.jpg</t>
         </is>
       </c>
       <c r="I328" t="inlineStr">
@@ -16791,7 +16801,7 @@
       </c>
       <c r="H329" t="inlineStr">
         <is>
-          <t xml:space="preserve">avene-tres-haute-protection-cream-spf50-mineral-3282779355773.jpg</t>
+          <t xml:space="preserve">sunscreens/avene-tres-haute-protection-cream-spf50-mineral-3282779355773.jpg</t>
         </is>
       </c>
       <c r="I329" t="inlineStr">
@@ -16841,7 +16851,7 @@
       </c>
       <c r="H330" t="inlineStr">
         <is>
-          <t xml:space="preserve">avene-tres-haute-protection-cream-spf50-teinte-3282770149524.jpg</t>
+          <t xml:space="preserve">sunscreens/avene-tres-haute-protection-cream-spf50-teinte-3282770149524.jpg</t>
         </is>
       </c>
       <c r="I330" t="inlineStr">
@@ -16886,7 +16896,7 @@
       </c>
       <c r="H331" t="inlineStr">
         <is>
-          <t xml:space="preserve">avene-tres-haute-protection-intense-fluid-spf50-150ml-3282770141214.jpg</t>
+          <t xml:space="preserve">sunscreens/avene-tres-haute-protection-intense-fluid-spf50-150ml-3282770141214.jpg</t>
         </is>
       </c>
       <c r="I331" t="inlineStr">
@@ -16936,7 +16946,7 @@
       </c>
       <c r="H332" t="inlineStr">
         <is>
-          <t xml:space="preserve">avene-tres-haute-protection-lait-spf50-mineral-100ml-3282779355872.jpg</t>
+          <t xml:space="preserve">sunscreens/avene-tres-haute-protection-lait-spf50-mineral-100ml-3282779355872.jpg</t>
         </is>
       </c>
       <c r="I332" t="inlineStr">
@@ -16986,7 +16996,7 @@
       </c>
       <c r="H333" t="inlineStr">
         <is>
-          <t xml:space="preserve">avene-tres-haute-protection-sport-spf50-100ml-3282770101362.jpg</t>
+          <t xml:space="preserve">sunscreens/avene-tres-haute-protection-sport-spf50-100ml-3282770101362.jpg</t>
         </is>
       </c>
       <c r="I333" t="inlineStr">
@@ -17036,7 +17046,7 @@
       </c>
       <c r="H334" t="inlineStr">
         <is>
-          <t xml:space="preserve">avene-tres-haute-protection-stick-spf50-20gr-3282770207576.jpg</t>
+          <t xml:space="preserve">sunscreens/avene-tres-haute-protection-stick-spf50-20gr-3282770207576.jpg</t>
         </is>
       </c>
       <c r="I334" t="inlineStr">
@@ -17086,7 +17096,7 @@
       </c>
       <c r="H335" t="inlineStr">
         <is>
-          <t xml:space="preserve">avene-ultra-fluid-invisible-spf50-50ml-3282770392654.jpg</t>
+          <t xml:space="preserve">sunscreens/avene-ultra-fluid-invisible-spf50-50ml-3282770392654.jpg</t>
         </is>
       </c>
       <c r="I335" t="inlineStr">
@@ -17141,7 +17151,7 @@
       </c>
       <c r="H336" t="inlineStr">
         <is>
-          <t xml:space="preserve">avene-ultra-fluid-oil-control-spf50-50ml-3282770397376.jpg</t>
+          <t xml:space="preserve">sunscreens/avene-ultra-fluid-oil-control-spf50-50ml-3282770397376.jpg</t>
         </is>
       </c>
       <c r="I336" t="inlineStr">
@@ -17191,7 +17201,7 @@
       </c>
       <c r="H337" t="inlineStr">
         <is>
-          <t xml:space="preserve">avene-ultra-fluid-perfect-spf50-50ml-3282770392692.jpg</t>
+          <t xml:space="preserve">sunscreens/avene-ultra-fluid-perfect-spf50-50ml-3282770392692.jpg</t>
         </is>
       </c>
       <c r="I337" t="inlineStr">
@@ -17241,7 +17251,7 @@
       </c>
       <c r="H338" t="inlineStr">
         <is>
-          <t xml:space="preserve">avene-ultra-fluid-radiance-spf50-50ml-3282770397697.jpg</t>
+          <t xml:space="preserve">sunscreens/avene-ultra-fluid-radiance-spf50-50ml-3282770397697.jpg</t>
         </is>
       </c>
       <c r="I338" t="inlineStr">
@@ -17296,7 +17306,7 @@
       </c>
       <c r="H339" t="inlineStr">
         <is>
-          <t xml:space="preserve">ducray-melascreen-protect-fluid-spf50-2x50ml-40-2-3282779371339.jpg</t>
+          <t xml:space="preserve">sunscreens/ducray-melascreen-protect-fluid-spf50-2x50ml-40-2-3282779371339.jpg</t>
         </is>
       </c>
       <c r="I339" t="inlineStr">
@@ -17351,7 +17361,7 @@
       </c>
       <c r="H340" t="inlineStr">
         <is>
-          <t xml:space="preserve">ducray-melascreen-teinte-fluid-spf50-30ml-3282770399653.jpg</t>
+          <t xml:space="preserve">sunscreens/ducray-melascreen-teinte-fluid-spf50-30ml-3282770399653.jpg</t>
         </is>
       </c>
       <c r="I340" t="inlineStr">
@@ -17406,7 +17416,7 @@
       </c>
       <c r="H341" t="inlineStr">
         <is>
-          <t xml:space="preserve">ducray-melascreen-anti-taches-cream-spf50-50ml-3282770389296.jpg</t>
+          <t xml:space="preserve">sunscreens/ducray-melascreen-anti-taches-cream-spf50-50ml-3282770389296.jpg</t>
         </is>
       </c>
       <c r="I341" t="inlineStr">
@@ -17461,7 +17471,7 @@
       </c>
       <c r="H342" t="inlineStr">
         <is>
-          <t xml:space="preserve">ducray-melascreen-anti-taches-fluid-spf50-50ml-3282770389272.jpg</t>
+          <t xml:space="preserve">sunscreens/ducray-melascreen-anti-taches-fluid-spf50-50ml-3282770389272.jpg</t>
         </is>
       </c>
       <c r="I342" t="inlineStr">
@@ -17516,7 +17526,7 @@
       </c>
       <c r="H343" t="inlineStr">
         <is>
-          <t xml:space="preserve">svr-sun-secure-blur-cream-spf50-50ml-teinte-3662361003167.jpg</t>
+          <t xml:space="preserve">sunscreens/svr-sun-secure-blur-cream-spf50-50ml-teinte-3662361003167.jpg</t>
         </is>
       </c>
       <c r="I343" t="inlineStr">
@@ -17566,7 +17576,7 @@
       </c>
       <c r="H344" t="inlineStr">
         <is>
-          <t xml:space="preserve">svr-sun-secure-blur-cream-spf50-50ml-3662361003150.jpg</t>
+          <t xml:space="preserve">sunscreens/svr-sun-secure-blur-cream-spf50-50ml-3662361003150.jpg</t>
         </is>
       </c>
       <c r="I344" t="inlineStr">
@@ -17616,7 +17626,7 @@
       </c>
       <c r="H345" t="inlineStr">
         <is>
-          <t xml:space="preserve">svr-sun-secure-blur-cream-spf50-mousse-50ml-3662361002597.jpg</t>
+          <t xml:space="preserve">sunscreens/svr-sun-secure-blur-cream-spf50-mousse-50ml-3662361002597.jpg</t>
         </is>
       </c>
       <c r="I345" t="inlineStr">
@@ -17666,7 +17676,7 @@
       </c>
       <c r="H346" t="inlineStr">
         <is>
-          <t xml:space="preserve">svr-sun-secure-brume-spray-spf50-200ml-3662361001699.jpg</t>
+          <t xml:space="preserve">sunscreens/svr-sun-secure-brume-spray-spf50-200ml-3662361001699.jpg</t>
         </is>
       </c>
       <c r="I346" t="inlineStr">
@@ -17716,7 +17726,7 @@
       </c>
       <c r="H347" t="inlineStr">
         <is>
-          <t xml:space="preserve">svr-sun-secure-cream-spf50-50ml-3662361001705.jpg</t>
+          <t xml:space="preserve">sunscreens/svr-sun-secure-cream-spf50-50ml-3662361001705.jpg</t>
         </is>
       </c>
       <c r="I347" t="inlineStr">
@@ -17766,7 +17776,7 @@
       </c>
       <c r="H348" t="inlineStr">
         <is>
-          <t xml:space="preserve">svr-sun-secure-spray-spf50-eau-solaire-200ml-3662361001293.jpg</t>
+          <t xml:space="preserve">sunscreens/svr-sun-secure-spray-spf50-eau-solaire-200ml-3662361001293.jpg</t>
         </is>
       </c>
       <c r="I348" t="inlineStr">
@@ -17816,7 +17826,7 @@
       </c>
       <c r="H349" t="inlineStr">
         <is>
-          <t xml:space="preserve">svr-sun-secure-gel-spf50-extreme-50ml-3662361002603.jpg</t>
+          <t xml:space="preserve">sunscreens/svr-sun-secure-gel-spf50-extreme-50ml-3662361002603.jpg</t>
         </is>
       </c>
       <c r="I349" t="inlineStr">
@@ -17866,7 +17876,7 @@
       </c>
       <c r="H350" t="inlineStr">
         <is>
-          <t xml:space="preserve">svr-sun-secure-spray-hydratant-spf50-200ml-3662361002146.jpg</t>
+          <t xml:space="preserve">sunscreens/svr-sun-secure-spray-hydratant-spf50-200ml-3662361002146.jpg</t>
         </is>
       </c>
       <c r="I350" t="inlineStr">
@@ -17916,7 +17926,7 @@
       </c>
       <c r="H351" t="inlineStr">
         <is>
-          <t xml:space="preserve">svr-sun-secure-lait-spray-spf50-200ml-3662361002559.jpg</t>
+          <t xml:space="preserve">sunscreens/svr-sun-secure-lait-spray-spf50-200ml-3662361002559.jpg</t>
         </is>
       </c>
       <c r="I351" t="inlineStr">
@@ -17966,7 +17976,7 @@
       </c>
       <c r="H352" t="inlineStr">
         <is>
-          <t xml:space="preserve">svr-sun-secure-huile-spray-seche-spf50-200ml-3662361001736.jpg</t>
+          <t xml:space="preserve">sunscreens/svr-sun-secure-huile-spray-seche-spf50-200ml-3662361001736.jpg</t>
         </is>
       </c>
       <c r="I352" t="inlineStr">
@@ -18016,7 +18026,7 @@
       </c>
       <c r="H353" t="inlineStr">
         <is>
-          <t xml:space="preserve">svr-sun-secure-lait-spf50-250ml-3662361001743.jpg</t>
+          <t xml:space="preserve">sunscreens/svr-sun-secure-lait-spf50-250ml-3662361001743.jpg</t>
         </is>
       </c>
       <c r="I353" t="inlineStr">
@@ -18066,7 +18076,7 @@
       </c>
       <c r="H354" t="inlineStr">
         <is>
-          <t xml:space="preserve">svr-sun-secure-fluid-spf50-50ml-3662361001729.jpg</t>
+          <t xml:space="preserve">sunscreens/svr-sun-secure-fluid-spf50-50ml-3662361001729.jpg</t>
         </is>
       </c>
       <c r="I354" t="inlineStr">
@@ -18116,7 +18126,7 @@
       </c>
       <c r="H355" t="inlineStr">
         <is>
-          <t xml:space="preserve">isdin-eryfotona-ak-nmsc-fluid-spf100-50ml-8470001658531.jpg</t>
+          <t xml:space="preserve">sunscreens/isdin-eryfotona-ak-nmsc-fluid-spf100-50ml-8470001658531.jpg</t>
         </is>
       </c>
       <c r="I355" t="inlineStr">
@@ -18166,7 +18176,7 @@
       </c>
       <c r="H356" t="inlineStr">
         <is>
-          <t xml:space="preserve">isdin-fotoprotector-fusion-water-spf50-color-50ml-8470001878199.jpg</t>
+          <t xml:space="preserve">sunscreens/isdin-fotoprotector-fusion-water-spf50-color-50ml-8470001878199.jpg</t>
         </is>
       </c>
       <c r="I356" t="inlineStr">
@@ -18211,7 +18221,7 @@
       </c>
       <c r="H357" t="inlineStr">
         <is>
-          <t xml:space="preserve">isdin-fotoprotector-fusion-water-spf50-magic-light-8429420231504.jpg</t>
+          <t xml:space="preserve">sunscreens/isdin-fotoprotector-fusion-water-spf50-magic-light-8429420231504.jpg</t>
         </is>
       </c>
       <c r="I357" t="inlineStr">
@@ -18261,7 +18271,7 @@
       </c>
       <c r="H358" t="inlineStr">
         <is>
-          <t xml:space="preserve">isdin-fotoprotector-pediatrics-spray-spf50-250ml-8429420188419.jpg</t>
+          <t xml:space="preserve">sunscreens/isdin-fotoprotector-pediatrics-spray-spf50-250ml-8429420188419.jpg</t>
         </is>
       </c>
       <c r="I358" t="inlineStr">
@@ -18311,7 +18321,7 @@
       </c>
       <c r="H359" t="inlineStr">
         <is>
-          <t xml:space="preserve">isdin-fotoultra-fusion-fluid-active-unify-spf50-50ml-8470001710529.jpg</t>
+          <t xml:space="preserve">sunscreens/isdin-fotoultra-fusion-fluid-active-unify-spf50-50ml-8470001710529.jpg</t>
         </is>
       </c>
       <c r="I359" t="inlineStr">
@@ -18366,7 +18376,7 @@
       </c>
       <c r="H360" t="inlineStr">
         <is>
-          <t xml:space="preserve">isdin-fotoultra-fusion-fluid-spot-prevent-spf50-50ml-8470001631688.jpg</t>
+          <t xml:space="preserve">sunscreens/isdin-fotoultra-fusion-fluid-spot-prevent-spf50-50ml-8470001631688.jpg</t>
         </is>
       </c>
       <c r="I360" t="inlineStr">
@@ -18421,7 +18431,7 @@
       </c>
       <c r="H361" t="inlineStr">
         <is>
-          <t xml:space="preserve">isdin-fotoultra-fusion-water-fluid-age-repair-spf50-color-8429420206014.jpg</t>
+          <t xml:space="preserve">sunscreens/isdin-fotoultra-fusion-water-fluid-age-repair-spf50-color-8429420206014.jpg</t>
         </is>
       </c>
       <c r="I361" t="inlineStr">
@@ -18461,7 +18471,7 @@
       </c>
       <c r="H362" t="inlineStr">
         <is>
-          <t xml:space="preserve">isdin-fotoultra-redness-control-spf50-50ml-8429420245297.jpg</t>
+          <t xml:space="preserve">sunscreens/isdin-fotoultra-redness-control-spf50-50ml-8429420245297.jpg</t>
         </is>
       </c>
       <c r="I362" t="inlineStr">

</xml_diff>

<commit_message>
Seasonal images + Greek descriptions (51/101 enriched)
</commit_message>
<xml_diff>
--- a/catalog.xlsx
+++ b/catalog.xlsx
@@ -15884,6 +15884,11 @@
           <t xml:space="preserve">Avène (Pierre Fabre)</t>
         </is>
       </c>
+      <c r="H311" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sunscreens/avene-enfant-haute-protection-spray-spf30-antioxydant-200ml-3282779402934.webp</t>
+        </is>
+      </c>
       <c r="I311" t="inlineStr">
         <is>
           <t xml:space="preserve">2200038064</t>

</xml_diff>

<commit_message>
Frezyderm: full scrape + tighter matcher + re-synced images
</commit_message>
<xml_diff>
--- a/catalog.xlsx
+++ b/catalog.xlsx
@@ -3351,7 +3351,7 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t xml:space="preserve">sunscreens/frezyderm-ac-norm-sunscreen-fluid-tinted-spf50-50ml-5202888400131.jpg</t>
+          <t xml:space="preserve">frezyderm/ac-norm-sun-screen-fluid-tinted-spf-50-5202888400131.jpg</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -3401,7 +3401,7 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t xml:space="preserve">sunscreens/frezyderm-ac-norm-sunscreen-fluid-spf50-50ml-5202888400025.jpg</t>
+          <t xml:space="preserve">frezyderm/ac-norm-sun-screen-fluid-spf-50-5202888400025.jpg</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -3456,7 +3456,7 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t xml:space="preserve">sunscreens/frezyderm-active-sun-cream-face-spf30-50ml-5202888400087.jpg</t>
+          <t xml:space="preserve">frezyderm/sun-screen-velvet-face-spf-30-5202888400087.jpg</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -3511,7 +3511,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t xml:space="preserve">sunscreens/frezyderm-active-sun-fluid-face-spf50-50ml-5202888400032.jpg</t>
+          <t xml:space="preserve">frezyderm/ac-norm-sun-screen-fluid-spf-50-5202888400032.jpg</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -3566,7 +3566,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t xml:space="preserve">sunscreens/frezyderm-active-sun-foundation-body-spf30-75ml-5202888400063.jpg</t>
+          <t xml:space="preserve">frezyderm/active-sun-screen-face-foundation-spf-30-5202888400063.jpg</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -3621,7 +3621,7 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t xml:space="preserve">sunscreens/frezyderm-active-sun-cream-face-spf50-50ml-5202888400094.jpg</t>
+          <t xml:space="preserve">frezyderm/ac-norm-sun-screen-fluid-spf-50-5202888400094.jpg</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -3681,7 +3681,7 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t xml:space="preserve">sunscreens/frezyderm-active-sun-cream-sensitive-face-body-spf50-5202888400056.jpg</t>
+          <t xml:space="preserve">frezyderm/active-sun-screen-sensitive-face-body-spf-50-5202888400056.jpg</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -3736,7 +3736,7 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t xml:space="preserve">sunscreens/frezyderm-active-sun-cream-tinted-face-spf50-5202888400100.jpg</t>
+          <t xml:space="preserve">frezyderm/active-sun-screen-cream-spray-spf-50-5202888400100.jpg</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -3791,7 +3791,7 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t xml:space="preserve">sunscreens/frezyderm-active-sun-fluid-tinted-face-spf50-5202888400049.jpg</t>
+          <t xml:space="preserve">frezyderm/ac-norm-sun-screen-fluid-spf-50-5202888400049.jpg</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -3841,7 +3841,7 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t xml:space="preserve">sunscreens/frezyderm-active-sun-foundation-face-spf30-30ml-5202888400070.jpg</t>
+          <t xml:space="preserve">frezyderm/active-sun-screen-face-foundation-spf-30-5202888400070.jpg</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -3896,7 +3896,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t xml:space="preserve">sunscreens/frezyderm-active-sun-lipbalm-spf50-15ml-5202888400018.jpg</t>
+          <t xml:space="preserve">frezyderm/active-sun-screen-lip-balm-spf-50-5202888400018.jpg</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -3946,7 +3946,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t xml:space="preserve">sunscreens/frezyderm-anti-thermal-water-mist-300ml-5202888222368.jpg</t>
+          <t xml:space="preserve">frezyderm/anti-thermal-spring-sea-water-mist-5202888222368.jpg</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -3996,7 +3996,7 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t xml:space="preserve">sunscreens/frezyderm-baby-suncare-spf25-lotion-100ml-5202888221262.jpg</t>
+          <t xml:space="preserve">frezyderm/baby-sun-care-spf-25-5202888221262.jpg</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -4051,7 +4051,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t xml:space="preserve">sunscreens/frezyderm-bronze-water-color-mist-300ml-5202888222382.jpg</t>
+          <t xml:space="preserve">frezyderm/anti-thermal-spring-sea-water-mist-5202888222382.jpg</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -4101,7 +4101,7 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t xml:space="preserve">sunscreens/frezyderm-infant-suncare-lotion-spf50-100ml-5202888271212.jpg</t>
+          <t xml:space="preserve">frezyderm/infant-sun-care-spf-50-5202888271212.jpg</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -4156,7 +4156,7 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t xml:space="preserve">sunscreens/frezyderm-kids-sunnip-lotion-spf50-150ml-25-5202888222436.jpg</t>
+          <t xml:space="preserve">frezyderm/ac-norm-sun-screen-fluid-spf-50-5202888222436.jpg</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -4211,7 +4211,7 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t xml:space="preserve">sunscreens/frezyderm-kids-suncare-lotion-spf50-175ml-5202888222429.jpg</t>
+          <t xml:space="preserve">frezyderm/kids-sun-care-spf-50-wet-skin-spray-5202888222429.jpg</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -4266,7 +4266,7 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t xml:space="preserve">sunscreens/frezyderm-kids-wetskin-spray-spf50-200ml-5202888221279.jpg</t>
+          <t xml:space="preserve">frezyderm/kids-sun-care-spf-50-wet-skin-spray-5202888221279.jpg</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
@@ -4361,7 +4361,7 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t xml:space="preserve">sunscreens/frezyderm-sea-side-dry-mist-spf50-300ml-5202888222375.jpg</t>
+          <t xml:space="preserve">frezyderm/sea-side-dry-mist-spf-50-5202888222375.jpg</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -4411,7 +4411,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t xml:space="preserve">sunscreens/frezyderm-self-tan-body-shape-150ml-5202888222283.jpg</t>
+          <t xml:space="preserve">frezyderm/self-tan-body-shape-5202888222283.jpg</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -4456,7 +4456,7 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t xml:space="preserve">sunscreens/frezyderm-sunscreen-after-sun-mousse-150ml-5202888102226.jpg</t>
+          <t xml:space="preserve">frezyderm/sun-screen-mousse-spf-30-5202888102226.jpg</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
@@ -4506,7 +4506,7 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t xml:space="preserve">sunscreens/frezyderm-sunscreen-cream-spray-kids-spf50-275ml-5202888222450.jpg</t>
+          <t xml:space="preserve">frezyderm/baby-sun-care-spf-50-5202888222450.jpg</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -4556,7 +4556,7 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t xml:space="preserve">sunscreens/frezyderm-sunscreen-on-the-move-spray-spf50-75ml-5202888222443.jpg</t>
+          <t xml:space="preserve">frezyderm/sun-screen-on-the-move-spf-50-5202888222443.jpg</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
@@ -4606,7 +4606,7 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t xml:space="preserve">sunscreens/frezyderm-sunscreen-tan-accelerator-cream-spf10-150ml-5202888102592.jpg</t>
+          <t xml:space="preserve">frezyderm/sun-screen-tan-accelerator-spf-10-5202888102592.jpg</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -4656,7 +4656,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t xml:space="preserve">sunscreens/frezyderm-sunscreen-cream-to-powder-spf50-50ml-5202888400124.jpg</t>
+          <t xml:space="preserve">frezyderm/sun-screen-cream-to-powder-spf-50-5202888400124.jpg</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -4706,7 +4706,7 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t xml:space="preserve">sunscreens/frezyderm-sunscreen-fluid-to-powder-spf50-50ml-5202888400117.png</t>
+          <t xml:space="preserve">frezyderm/sun-screen-fluid-to-powder-spf-50-5202888400117.jpg</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -4756,7 +4756,7 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t xml:space="preserve">sunscreens/frezyderm-sunscreen-invisible-spray-spf50-200ml-5202888222405.jpg</t>
+          <t xml:space="preserve">frezyderm/sun-screen-invisible-spray-spf-50-5202888222405.jpg</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -4806,7 +4806,7 @@
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t xml:space="preserve">sunscreens/frezyderm-sunscreen-mousse-spf50-200ml-5202888222467.jpg</t>
+          <t xml:space="preserve">frezyderm/sun-screen-mousse-spf-50-5202888222467.jpg</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
@@ -4856,7 +4856,7 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t xml:space="preserve">sunscreens/frezyderm-sunscreen-mousse-spf30-200ml-5202888222412.jpg</t>
+          <t xml:space="preserve">frezyderm/sun-screen-mousse-spf-30-5202888222412.jpg</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
@@ -4906,7 +4906,7 @@
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t xml:space="preserve">sunscreens/frezyderm-sunscreen-spray-anti-seb-spf30-5202888102516.jpg</t>
+          <t xml:space="preserve">frezyderm/sun-screen-anti-seb-spray-spf-30-5202888102516.jpg</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
@@ -4956,7 +4956,7 @@
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t xml:space="preserve">sunscreens/frezyderm-sunscreen-velvet-color-cream-spf50-5202888222351.jpg</t>
+          <t xml:space="preserve">frezyderm/sun-screen-color-velvet-face-spf-50-5202888222351.jpg</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
@@ -5006,7 +5006,7 @@
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t xml:space="preserve">sunscreens/frezyderm-sunscreen-velvet-color-cream-spf30-5202888222399.jpg</t>
+          <t xml:space="preserve">frezyderm/sun-screen-color-velvet-face-spf-50-5202888222399.jpg</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
@@ -5056,7 +5056,7 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t xml:space="preserve">sunscreens/frezyderm-sunscreen-velvet-cream-face-spf30-5202888222306.jpg</t>
+          <t xml:space="preserve">frezyderm/sun-screen-velvet-face-spf-30-5202888222306.jpg</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
@@ -5106,7 +5106,7 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t xml:space="preserve">sunscreens/frezyderm-sunscreen-velvet-cream-face-spf50-5202888222290.jpg</t>
+          <t xml:space="preserve">frezyderm/sun-screen-velvet-face-spf-50-5202888222290.jpg</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -5156,7 +5156,7 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t xml:space="preserve">sunscreens/frezyderm-sunscreen-velvet-lotion-body-spf50-5202888222313.jpg</t>
+          <t xml:space="preserve">frezyderm/sun-screen-velvet-face-spf-50-5202888222313.jpg</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">

</xml_diff>

<commit_message>
Frezyderm: filled missing from pharmacies
</commit_message>
<xml_diff>
--- a/catalog.xlsx
+++ b/catalog.xlsx
@@ -3736,7 +3736,7 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm/active-sun-screen-cream-spray-spf-50-5202888400100.jpg</t>
+          <t xml:space="preserve">frezyderm/active-sun-screen-tinted-face-cream-spf50-50ml-pharm24-gr-5202888400100.jpg</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -4156,7 +4156,7 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm/ac-norm-sun-screen-fluid-spf-50-5202888222436.jpg</t>
+          <t xml:space="preserve">frezyderm/for-kids-sun-nip-lotion-spf50-175ml-pharm24-gr-5202888222436.jpg</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -4316,7 +4316,7 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t xml:space="preserve">sunscreens/frezyderm-proflamine-cream-40ml-5202888261015.jpg</t>
+          <t xml:space="preserve">frezyderm/proflamine-40ml-pharm24-gr-5202888261015.jpg</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -4506,7 +4506,7 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm/baby-sun-care-spf-50-5202888222450.jpg</t>
+          <t xml:space="preserve">frezyderm/kids-sun-care-cream-spray-spf50-275ml-pharm24-gr-5202888222450.jpg</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -5251,7 +5251,7 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t xml:space="preserve">sunscreens/frezyderm-icy-after-sun-hydrogel-200ml-5202888222474.jpg</t>
+          <t xml:space="preserve">frezyderm/icy-after-sun-relieving-cooling-hydrogel-face-body-200ml-pharm24-gr-5202888222474.jpg</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">

</xml_diff>

<commit_message>
Frezyderm: excluded Boosters + Promo bundles from catalogue
</commit_message>
<xml_diff>
--- a/catalog.xlsx
+++ b/catalog.xlsx
@@ -4506,7 +4506,7 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm/kids-sun-care-cream-spray-spf50-275ml-pharm24-gr-5202888222450.jpg</t>
+          <t xml:space="preserve">frezyderm/kids-sun-care-cream-spray-water-resistant-spf50-275ml-ofarmakopoiosmou-gr-5202888222450.jpg</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -5251,7 +5251,7 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t xml:space="preserve">frezyderm/icy-after-sun-relieving-cooling-hydrogel-face-body-200ml-pharm24-gr-5202888222474.jpg</t>
+          <t xml:space="preserve">frezyderm/icy-after-sun-face-body-200ml-online-pharmacy-ofarmakopoiosmou-gr-5202888222474.jpg</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">

</xml_diff>